<commit_message>
V2 version and fixes from V1. Can pull historic data, improve UI, add a ticker not found and documented use of SEC Edgar User-Agent requirement.
</commit_message>
<xml_diff>
--- a/DCF_Model_Sample.xlsx
+++ b/DCF_Model_Sample.xlsx
@@ -1,19 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Guide" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Stock Search" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Assumptions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Income Statement" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="WACC" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="DCF Valuation" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Sensitivity" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stock Search" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income Statement" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WACC" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF Valuation" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reverse DCF" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Price" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28,7 +31,7 @@
     <numFmt numFmtId="166" formatCode="0.0"/>
     <numFmt numFmtId="167" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -137,12 +140,18 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00606060"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="8"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -182,6 +191,26 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C00000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00375623"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -229,9 +258,7 @@
     </border>
     <border>
       <left/>
-      <right style="thin">
-        <color rgb="008EA9C1"/>
-      </right>
+      <right/>
       <top style="thin">
         <color rgb="008EA9C1"/>
       </top>
@@ -242,7 +269,9 @@
     </border>
     <border>
       <left/>
-      <right/>
+      <right style="thin">
+        <color rgb="008EA9C1"/>
+      </right>
       <top style="thin">
         <color rgb="008EA9C1"/>
       </top>
@@ -255,7 +284,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -383,10 +412,13 @@
     <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="166" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -416,7 +448,7 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -431,8 +463,47 @@
     <xf numFmtId="165" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="13" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="13" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="13" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -510,18 +581,18 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Projected FCFF  (USD $M)</a:t>
+              <a:t>FCF Projection  (USD $M)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -531,17 +602,24 @@
       <barChart>
         <barDir val="col"/>
         <grouping val="clustered"/>
+        <varyColors val="1"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill>
-              <a:srgbClr val="2E4170"/>
-            </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <dLbls>
+            <numFmt formatCode="#,##0"/>
+            <showLegendKey val="0"/>
+            <showVal val="1"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+            <showBubbleSize val="0"/>
+          </dLbls>
           <cat>
             <numRef>
               <f>'Income Statement'!$F$4:$O$4</f>
@@ -549,182 +627,11 @@
           </cat>
           <val>
             <numRef>
-              <f>'Income Statement'!$F$29</f>
+              <f>'Income Statement'!$F$29:$O$29</f>
             </numRef>
           </val>
         </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Income Statement'!$F$4:$O$4</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Income Statement'!$G$29</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="2"/>
-          <order val="2"/>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Income Statement'!$F$4:$O$4</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Income Statement'!$H$29</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="3"/>
-          <order val="3"/>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Income Statement'!$F$4:$O$4</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Income Statement'!$I$29</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="4"/>
-          <order val="4"/>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Income Statement'!$F$4:$O$4</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Income Statement'!$J$29</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="5"/>
-          <order val="5"/>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Income Statement'!$F$4:$O$4</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Income Statement'!$K$29</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="6"/>
-          <order val="6"/>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Income Statement'!$F$4:$O$4</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Income Statement'!$L$29</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="7"/>
-          <order val="7"/>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Income Statement'!$F$4:$O$4</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Income Statement'!$M$29</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="8"/>
-          <order val="8"/>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Income Statement'!$F$4:$O$4</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Income Statement'!$N$29</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="9"/>
-          <order val="9"/>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Income Statement'!$F$4:$O$4</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Income Statement'!$O$29</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="150"/>
+        <gapWidth val="30"/>
         <axId val="10"/>
         <axId val="100"/>
       </barChart>
@@ -733,9 +640,11 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="low"/>
         <crossAx val="100"/>
         <lblOffset val="100"/>
       </catAx>
@@ -745,12 +654,11 @@
           <orientation val="minMax"/>
         </scaling>
         <axPos val="l"/>
-        <majorGridlines/>
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -766,9 +674,6 @@
         <crossAx val="10"/>
       </valAx>
     </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
@@ -776,7 +681,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>1</col>
@@ -784,16 +689,16 @@
       <row>32</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8640000" cy="3600000"/>
+    <ext cx="8640000" cy="4680000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1092,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:C10"/>
+  <dimension ref="B1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1110,77 +1015,430 @@
     <row r="2" ht="16" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Built 2026-05-25  |  Gold cells = inputs  |  White cells = formulas</t>
+          <t xml:space="preserve">  Built 2026-06-02  |  Gold cells = inputs  |  White cells = formulas</t>
         </is>
       </c>
     </row>
     <row r="4" ht="14" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  [Stock Search]  Enter ticker in B5. Microsoft 365: Data &gt; Stocks to link live data.</t>
-        </is>
-      </c>
-      <c r="C4" s="61" t="n"/>
+          <t xml:space="preserve">  [Stock Search]  One command to build and populate — pick your stock and date:</t>
+        </is>
+      </c>
+      <c r="C4" s="73" t="n"/>
     </row>
     <row r="5" ht="13" customHeight="1">
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">       Or run:  python build_dcf.py AAPL  to build and auto-fill in one step.</t>
-        </is>
-      </c>
-      <c r="C5" s="61" t="n"/>
-    </row>
-    <row r="6" ht="14" customHeight="1">
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  [Assumptions]  Edit all gold cells. Revenue growth, margins, WACC inputs, terminal value.</t>
-        </is>
-      </c>
-      <c r="C6" s="61" t="n"/>
-    </row>
-    <row r="7" ht="14" customHeight="1">
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  [Income Statement]  Historical (grey) + 10-year projection. FCF computed automatically.</t>
-        </is>
-      </c>
-      <c r="C7" s="61" t="n"/>
-    </row>
-    <row r="8" ht="14" customHeight="1">
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  [WACC]  Cost of equity (CAPM), cost of debt, capital structure -&gt; WACC.</t>
-        </is>
-      </c>
-      <c r="C8" s="61" t="n"/>
+          <t xml:space="preserve">         python build_dcf.py AAPL                     (live data)</t>
+        </is>
+      </c>
+      <c r="C5" s="73" t="n"/>
+    </row>
+    <row r="6" ht="13" customHeight="1">
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">         python build_dcf.py AAPL --date 2020-03-23   (COVID crash low)</t>
+        </is>
+      </c>
+      <c r="C6" s="73" t="n"/>
+    </row>
+    <row r="7" ht="13" customHeight="1">
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">         python build_dcf.py AAPL --date 2008         (financial crisis)</t>
+        </is>
+      </c>
+      <c r="C7" s="73" t="n"/>
+    </row>
+    <row r="8" ht="13" customHeight="1">
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">       Microsoft 365: select B5 then Data &gt; Stocks to link live data.</t>
+        </is>
+      </c>
+      <c r="C8" s="73" t="n"/>
     </row>
     <row r="9" ht="14" customHeight="1">
       <c r="B9" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">  [Assumptions]  Edit all gold cells. Revenue growth, margins, WACC inputs, terminal value.</t>
+        </is>
+      </c>
+      <c r="C9" s="73" t="n"/>
+    </row>
+    <row r="10" ht="13" customHeight="1">
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">       To refresh data only:  python update_dcf.py AAPL  (keeps your thesis intact)</t>
+        </is>
+      </c>
+      <c r="C10" s="73" t="n"/>
+    </row>
+    <row r="11" ht="14" customHeight="1">
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  [Income Statement]  Historical (grey) + 10-year projection. FCF computed automatically.</t>
+        </is>
+      </c>
+      <c r="C11" s="73" t="n"/>
+    </row>
+    <row r="12" ht="14" customHeight="1">
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  [WACC]  Cost of equity (CAPM), cost of debt, capital structure -&gt; WACC.</t>
+        </is>
+      </c>
+      <c r="C12" s="73" t="n"/>
+    </row>
+    <row r="13" ht="14" customHeight="1">
+      <c r="B13" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">  [DCF Valuation]  Discounted FCFs + terminal value -&gt; Enterprise Value -&gt; Implied Price.</t>
         </is>
       </c>
-      <c r="C9" s="61" t="n"/>
-    </row>
-    <row r="10" ht="14" customHeight="1">
-      <c r="B10" s="5" t="inlineStr">
+      <c r="C13" s="73" t="n"/>
+    </row>
+    <row r="14" ht="14" customHeight="1">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  [Sensitivity]  Implied price vs WACC x terminal growth rate. Green = upside.</t>
         </is>
       </c>
-      <c r="C10" s="61" t="n"/>
+      <c r="C14" s="73" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="13">
+    <mergeCell ref="B13:C13"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B11:C11"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B14:C14"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B12:C12"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="004472C4"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:E20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="B1" s="20" t="inlineStr">
+        <is>
+          <t>PRICE TRACKER  -  Intraday Monitor</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="13" customHeight="1">
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Run  python update_dcf.py TICKER  to refresh. Gold cells = live data from Yahoo Finance. White = formulas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1">
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  COMPANY</t>
+        </is>
+      </c>
+      <c r="C4" s="72" t="n"/>
+      <c r="D4" s="72" t="n"/>
+      <c r="E4" s="73" t="n"/>
+    </row>
+    <row r="5" ht="17" customHeight="1">
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Ticker</t>
+        </is>
+      </c>
+      <c r="C5" s="41">
+        <f>'Stock Search'!B5</f>
+        <v/>
+      </c>
+      <c r="D5" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Company</t>
+        </is>
+      </c>
+      <c r="E5" s="41">
+        <f>'Stock Search'!D5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" ht="17" customHeight="1">
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Beta (1-yr vs S&amp;P 500)</t>
+        </is>
+      </c>
+      <c r="C6" s="38">
+        <f>Assumptions!C22</f>
+        <v/>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Last Updated</t>
+        </is>
+      </c>
+      <c r="E6" s="41">
+        <f>TEXT('Stock Search'!E5,"YYYY-MM-DD")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1">
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SESSION PRICES  (refreshed by update_dcf.py)</t>
+        </is>
+      </c>
+      <c r="C7" s="72" t="n"/>
+      <c r="D7" s="72" t="n"/>
+      <c r="E7" s="73" t="n"/>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="B8" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Open ($)</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="n">
+        <v>309.63</v>
+      </c>
+      <c r="D8" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Market Status</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>HISTORICAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="B9" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Current ($)</t>
+        </is>
+      </c>
+      <c r="C9" s="71">
+        <f>'Stock Search'!C5</f>
+        <v/>
+      </c>
+      <c r="D9" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Change from Open ($)</t>
+        </is>
+      </c>
+      <c r="E9" s="71">
+        <f>'Stock Search'!C5-C8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="17" customHeight="1">
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Session High ($)</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="n">
+        <v>310.94</v>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Session Low ($)</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="n">
+        <v>305.02</v>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="B11" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Change from Open (%)</t>
+        </is>
+      </c>
+      <c r="C11" s="24">
+        <f>IF(C8=0,0,('Stock Search'!C5-C8)/C8)</f>
+        <v/>
+      </c>
+      <c r="D11" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  High-Low Range ($)</t>
+        </is>
+      </c>
+      <c r="E11" s="71">
+        <f>C10-E10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="15" customHeight="1">
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  52-WEEK RANGE</t>
+        </is>
+      </c>
+      <c r="C12" s="72" t="n"/>
+      <c r="D12" s="72" t="n"/>
+      <c r="E12" s="73" t="n"/>
+    </row>
+    <row r="13" ht="17" customHeight="1">
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  52-Week High ($)</t>
+        </is>
+      </c>
+      <c r="C13" s="53">
+        <f>'Stock Search'!D8</f>
+        <v/>
+      </c>
+      <c r="D13" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  52-Week Low ($)</t>
+        </is>
+      </c>
+      <c r="E13" s="53">
+        <f>'Stock Search'!E8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="17" customHeight="1">
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  vs 52-Week High</t>
+        </is>
+      </c>
+      <c r="C14" s="34">
+        <f>IF(C13=0,0,('Stock Search'!C5-C13)/C13)</f>
+        <v/>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  vs 52-Week Low</t>
+        </is>
+      </c>
+      <c r="E14" s="34">
+        <f>IF(E13=0,0,('Stock Search'!C5-E13)/E13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="17" customHeight="1">
+      <c r="B15" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  52-Week Percentile  (100% = at 52W high)</t>
+        </is>
+      </c>
+      <c r="C15" s="55">
+        <f>IFERROR(('Stock Search'!C5-E13)/(C13-E13),0)</f>
+        <v/>
+      </c>
+      <c r="D15" s="72" t="n"/>
+      <c r="E15" s="73" t="n"/>
+    </row>
+    <row r="16" ht="15" customHeight="1">
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  BETA-ADJUSTED PERFORMANCE  (vs S&amp;P 500 today)</t>
+        </is>
+      </c>
+      <c r="C16" s="72" t="n"/>
+      <c r="D16" s="72" t="n"/>
+      <c r="E16" s="73" t="n"/>
+    </row>
+    <row r="17" ht="17" customHeight="1">
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  S&amp;P 500 Move Today (%)</t>
+        </is>
+      </c>
+      <c r="C17" s="21" t="n">
+        <v>0.0023</v>
+      </c>
+      <c r="D17" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  (auto-filled by update_dcf.py)</t>
+        </is>
+      </c>
+      <c r="E17" s="22" t="inlineStr"/>
+    </row>
+    <row r="18" ht="17" customHeight="1">
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Expected Move  (Beta x S&amp;P move)</t>
+        </is>
+      </c>
+      <c r="C18" s="34">
+        <f>Assumptions!C22*C17</f>
+        <v/>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Actual Move (vs open)</t>
+        </is>
+      </c>
+      <c r="E18" s="34">
+        <f>C11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="B19" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Alpha Today  (actual - expected)</t>
+        </is>
+      </c>
+      <c r="C19" s="24">
+        <f>C11-Assumptions!C22*C17</f>
+        <v/>
+      </c>
+      <c r="D19" s="72" t="n"/>
+      <c r="E19" s="73" t="n"/>
+    </row>
+    <row r="20" ht="14" customHeight="1">
+      <c r="B20" s="45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Alpha = actual stock move minus CAPM-predicted move (beta x market). Positive alpha = stock outperformed its risk-adjusted expectation today.</t>
+        </is>
+      </c>
+      <c r="C20" s="72" t="n"/>
+      <c r="D20" s="72" t="n"/>
+      <c r="E20" s="73" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="B16:E16"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B20:E20"/>
+    <mergeCell ref="C15:E15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1193,7 +1451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:E28"/>
+  <dimension ref="B1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1246,7 +1504,7 @@
         </is>
       </c>
       <c r="C5" s="10" t="n">
-        <v>308.82</v>
+        <v>306.31</v>
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
@@ -1255,7 +1513,7 @@
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-06-01 (historical)</t>
         </is>
       </c>
     </row>
@@ -1265,9 +1523,9 @@
           <t xml:space="preserve">  PRICE &amp; RANGE</t>
         </is>
       </c>
-      <c r="C7" s="62" t="n"/>
-      <c r="D7" s="62" t="n"/>
-      <c r="E7" s="61" t="n"/>
+      <c r="C7" s="72" t="n"/>
+      <c r="D7" s="72" t="n"/>
+      <c r="E7" s="73" t="n"/>
     </row>
     <row r="8" ht="17" customHeight="1">
       <c r="B8" s="12" t="inlineStr">
@@ -1276,13 +1534,13 @@
         </is>
       </c>
       <c r="C8" s="10" t="n">
-        <v>308.82</v>
+        <v>306.31</v>
       </c>
       <c r="D8" s="10" t="n">
-        <v>311.4</v>
+        <v>315</v>
       </c>
       <c r="E8" s="10" t="n">
-        <v>192.7</v>
+        <v>194.3</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
@@ -1291,9 +1549,9 @@
           <t xml:space="preserve">  SHARES &amp; MARKET CAP</t>
         </is>
       </c>
-      <c r="C9" s="62" t="n"/>
-      <c r="D9" s="62" t="n"/>
-      <c r="E9" s="61" t="n"/>
+      <c r="C9" s="72" t="n"/>
+      <c r="D9" s="72" t="n"/>
+      <c r="E9" s="73" t="n"/>
     </row>
     <row r="10" ht="17" customHeight="1">
       <c r="B10" s="12" t="inlineStr">
@@ -1302,13 +1560,13 @@
         </is>
       </c>
       <c r="C10" s="13" t="n">
-        <v>4535749.2</v>
+        <v>4498884</v>
       </c>
       <c r="D10" s="13" t="n">
         <v>14687.4</v>
       </c>
       <c r="E10" s="14" t="n">
-        <v>0.9983</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
@@ -1317,9 +1575,9 @@
           <t xml:space="preserve">  INCOME (TTM, $M)</t>
         </is>
       </c>
-      <c r="C11" s="62" t="n"/>
-      <c r="D11" s="62" t="n"/>
-      <c r="E11" s="61" t="n"/>
+      <c r="C11" s="72" t="n"/>
+      <c r="D11" s="72" t="n"/>
+      <c r="E11" s="73" t="n"/>
     </row>
     <row r="12" ht="17" customHeight="1">
       <c r="B12" s="12" t="inlineStr">
@@ -1328,13 +1586,13 @@
         </is>
       </c>
       <c r="C12" s="13" t="n">
-        <v>451442</v>
+        <v>416161</v>
       </c>
       <c r="D12" s="13" t="n">
-        <v>159976</v>
+        <v>144748</v>
       </c>
       <c r="E12" s="13" t="n">
-        <v>122575</v>
+        <v>112010</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
@@ -1343,9 +1601,9 @@
           <t xml:space="preserve">  BALANCE SHEET ($M)</t>
         </is>
       </c>
-      <c r="C13" s="62" t="n"/>
-      <c r="D13" s="62" t="n"/>
-      <c r="E13" s="61" t="n"/>
+      <c r="C13" s="72" t="n"/>
+      <c r="D13" s="72" t="n"/>
+      <c r="E13" s="73" t="n"/>
     </row>
     <row r="14" ht="17" customHeight="1">
       <c r="B14" s="12" t="inlineStr">
@@ -1354,10 +1612,10 @@
         </is>
       </c>
       <c r="C14" s="13" t="n">
-        <v>84711</v>
+        <v>98657</v>
       </c>
       <c r="D14" s="13" t="n">
-        <v>68507</v>
+        <v>35934</v>
       </c>
       <c r="E14" s="15">
         <f>C16-D16</f>
@@ -1370,9 +1628,9 @@
           <t xml:space="preserve">  VALUATION</t>
         </is>
       </c>
-      <c r="C15" s="62" t="n"/>
-      <c r="D15" s="62" t="n"/>
-      <c r="E15" s="61" t="n"/>
+      <c r="C15" s="72" t="n"/>
+      <c r="D15" s="72" t="n"/>
+      <c r="E15" s="73" t="n"/>
     </row>
     <row r="16" ht="17" customHeight="1">
       <c r="B16" s="12" t="inlineStr">
@@ -1381,13 +1639,13 @@
         </is>
       </c>
       <c r="C16" s="16" t="n">
-        <v>37.4</v>
+        <v>40.2</v>
       </c>
       <c r="D16" s="16" t="n">
-        <v>28.5</v>
+        <v>31.5</v>
       </c>
       <c r="E16" s="17" t="n">
-        <v>1.06</v>
+        <v>0.9399999999999999</v>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
@@ -1396,9 +1654,9 @@
           <t xml:space="preserve">  MICROSOFT 365 STOCKS DATA TYPE - INSTRUCTIONS</t>
         </is>
       </c>
-      <c r="C18" s="62" t="n"/>
-      <c r="D18" s="62" t="n"/>
-      <c r="E18" s="61" t="n"/>
+      <c r="C18" s="72" t="n"/>
+      <c r="D18" s="72" t="n"/>
+      <c r="E18" s="73" t="n"/>
     </row>
     <row r="19" ht="13" customHeight="1">
       <c r="B19" s="18" t="inlineStr">
@@ -1406,9 +1664,9 @@
           <t xml:space="preserve">  1. Type ticker in B5  (e.g. AAPL, MSFT, GOOGL, NVDA)</t>
         </is>
       </c>
-      <c r="C19" s="62" t="n"/>
-      <c r="D19" s="62" t="n"/>
-      <c r="E19" s="61" t="n"/>
+      <c r="C19" s="72" t="n"/>
+      <c r="D19" s="72" t="n"/>
+      <c r="E19" s="73" t="n"/>
     </row>
     <row r="20" ht="13" customHeight="1">
       <c r="B20" s="18" t="inlineStr">
@@ -1416,9 +1674,9 @@
           <t xml:space="preserve">  2. With B5 selected: click  Data  tab  &gt;  Stocks  button in ribbon</t>
         </is>
       </c>
-      <c r="C20" s="62" t="n"/>
-      <c r="D20" s="62" t="n"/>
-      <c r="E20" s="61" t="n"/>
+      <c r="C20" s="72" t="n"/>
+      <c r="D20" s="72" t="n"/>
+      <c r="E20" s="73" t="n"/>
     </row>
     <row r="21" ht="13" customHeight="1">
       <c r="B21" s="18" t="inlineStr">
@@ -1426,9 +1684,9 @@
           <t xml:space="preserve">  3. Excel converts the text to a linked Stocks data type (shows stock icon)</t>
         </is>
       </c>
-      <c r="C21" s="62" t="n"/>
-      <c r="D21" s="62" t="n"/>
-      <c r="E21" s="61" t="n"/>
+      <c r="C21" s="72" t="n"/>
+      <c r="D21" s="72" t="n"/>
+      <c r="E21" s="73" t="n"/>
     </row>
     <row r="22" ht="13" customHeight="1">
       <c r="B22" s="18" t="inlineStr">
@@ -1436,9 +1694,9 @@
           <t xml:space="preserve">  4. Click the icon to browse available fields, or type  =B5.Price  to extract any field</t>
         </is>
       </c>
-      <c r="C22" s="62" t="n"/>
-      <c r="D22" s="62" t="n"/>
-      <c r="E22" s="61" t="n"/>
+      <c r="C22" s="72" t="n"/>
+      <c r="D22" s="72" t="n"/>
+      <c r="E22" s="73" t="n"/>
     </row>
     <row r="23" ht="13" customHeight="1">
       <c r="B23" s="18" t="inlineStr">
@@ -1446,19 +1704,19 @@
           <t xml:space="preserve">  5. STOCKHISTORY(B5, start_date, end_date)  returns historical price table</t>
         </is>
       </c>
-      <c r="C23" s="62" t="n"/>
-      <c r="D23" s="62" t="n"/>
-      <c r="E23" s="61" t="n"/>
+      <c r="C23" s="72" t="n"/>
+      <c r="D23" s="72" t="n"/>
+      <c r="E23" s="73" t="n"/>
     </row>
     <row r="24" ht="13" customHeight="1">
       <c r="B24" s="18" t="inlineStr">
         <is>
-          <t>  </t>
-        </is>
-      </c>
-      <c r="C24" s="62" t="n"/>
-      <c r="D24" s="62" t="n"/>
-      <c r="E24" s="61" t="n"/>
+          <t xml:space="preserve">  </t>
+        </is>
+      </c>
+      <c r="C24" s="72" t="n"/>
+      <c r="D24" s="72" t="n"/>
+      <c r="E24" s="73" t="n"/>
     </row>
     <row r="25" ht="13" customHeight="1">
       <c r="B25" s="5" t="inlineStr">
@@ -1466,9 +1724,9 @@
           <t xml:space="preserve">  PYTHON AUTO-FILL (works with any Excel version):</t>
         </is>
       </c>
-      <c r="C25" s="62" t="n"/>
-      <c r="D25" s="62" t="n"/>
-      <c r="E25" s="61" t="n"/>
+      <c r="C25" s="72" t="n"/>
+      <c r="D25" s="72" t="n"/>
+      <c r="E25" s="73" t="n"/>
     </row>
     <row r="26" ht="13" customHeight="1">
       <c r="B26" s="19" t="inlineStr">
@@ -1476,32 +1734,22 @@
           <t xml:space="preserve">     pip install yfinance openpyxl</t>
         </is>
       </c>
-      <c r="C26" s="62" t="n"/>
-      <c r="D26" s="62" t="n"/>
-      <c r="E26" s="61" t="n"/>
+      <c r="C26" s="72" t="n"/>
+      <c r="D26" s="72" t="n"/>
+      <c r="E26" s="73" t="n"/>
     </row>
     <row r="27" ht="13" customHeight="1">
       <c r="B27" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">     python build_dcf.py AAPL   (build + fill in one step)</t>
-        </is>
-      </c>
-      <c r="C27" s="62" t="n"/>
-      <c r="D27" s="62" t="n"/>
-      <c r="E27" s="61" t="n"/>
-    </row>
-    <row r="28" ht="13" customHeight="1">
-      <c r="B28" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     python update_dcf.py AAPL  (refresh an existing model)</t>
-        </is>
-      </c>
-      <c r="C28" s="62" t="n"/>
-      <c r="D28" s="62" t="n"/>
-      <c r="E28" s="61" t="n"/>
+          <t xml:space="preserve">     python update_dcf.py AAPL</t>
+        </is>
+      </c>
+      <c r="C27" s="72" t="n"/>
+      <c r="D27" s="72" t="n"/>
+      <c r="E27" s="73" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="23">
+  <mergeCells count="22">
     <mergeCell ref="B9:E9"/>
     <mergeCell ref="B15:E15"/>
     <mergeCell ref="B24:E24"/>
@@ -1524,7 +1772,6 @@
     <mergeCell ref="B13:E13"/>
     <mergeCell ref="B10"/>
     <mergeCell ref="B19:E19"/>
-    <mergeCell ref="B28:E28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1567,9 +1814,9 @@
           <t xml:space="preserve">  COMPANY</t>
         </is>
       </c>
-      <c r="C4" s="62" t="n"/>
-      <c r="D4" s="62" t="n"/>
-      <c r="E4" s="61" t="n"/>
+      <c r="C4" s="72" t="n"/>
+      <c r="D4" s="72" t="n"/>
+      <c r="E4" s="73" t="n"/>
     </row>
     <row r="5" ht="17" customHeight="1">
       <c r="B5" s="18" t="inlineStr">
@@ -1622,7 +1869,7 @@
         </is>
       </c>
       <c r="C7" s="10" t="n">
-        <v>308.82</v>
+        <v>306.31</v>
       </c>
       <c r="D7" s="18" t="inlineStr">
         <is>
@@ -1640,7 +1887,7 @@
         </is>
       </c>
       <c r="C8" s="13" t="n">
-        <v>84711</v>
+        <v>98657</v>
       </c>
       <c r="D8" s="18" t="inlineStr">
         <is>
@@ -1648,7 +1895,7 @@
         </is>
       </c>
       <c r="E8" s="13" t="n">
-        <v>68507</v>
+        <v>35934</v>
       </c>
     </row>
     <row r="9" ht="17" customHeight="1">
@@ -1657,9 +1904,9 @@
           <t xml:space="preserve">  REVENUE GROWTH  (10-year projection ramp)</t>
         </is>
       </c>
-      <c r="C9" s="62" t="n"/>
-      <c r="D9" s="62" t="n"/>
-      <c r="E9" s="61" t="n"/>
+      <c r="C9" s="72" t="n"/>
+      <c r="D9" s="72" t="n"/>
+      <c r="E9" s="73" t="n"/>
     </row>
     <row r="10" ht="17" customHeight="1">
       <c r="B10" s="18" t="inlineStr">
@@ -1757,9 +2004,9 @@
           <t xml:space="preserve">  MARGIN ASSUMPTIONS</t>
         </is>
       </c>
-      <c r="C15" s="62" t="n"/>
-      <c r="D15" s="62" t="n"/>
-      <c r="E15" s="61" t="n"/>
+      <c r="C15" s="72" t="n"/>
+      <c r="D15" s="72" t="n"/>
+      <c r="E15" s="73" t="n"/>
     </row>
     <row r="16" ht="17" customHeight="1">
       <c r="B16" s="18" t="inlineStr">
@@ -1833,9 +2080,9 @@
           <t xml:space="preserve">  WACC INPUTS</t>
         </is>
       </c>
-      <c r="C20" s="62" t="n"/>
-      <c r="D20" s="62" t="n"/>
-      <c r="E20" s="61" t="n"/>
+      <c r="C20" s="72" t="n"/>
+      <c r="D20" s="72" t="n"/>
+      <c r="E20" s="73" t="n"/>
     </row>
     <row r="21" ht="17" customHeight="1">
       <c r="B21" s="18" t="inlineStr">
@@ -1844,7 +2091,7 @@
         </is>
       </c>
       <c r="C21" s="21" t="n">
-        <v>0.043</v>
+        <v>0.04475</v>
       </c>
       <c r="D21" s="18" t="inlineStr">
         <is>
@@ -1862,7 +2109,7 @@
         </is>
       </c>
       <c r="C22" s="17" t="n">
-        <v>1.06</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="D22" s="18" t="inlineStr">
         <is>
@@ -1910,9 +2157,9 @@
           <t xml:space="preserve">  TERMINAL VALUE</t>
         </is>
       </c>
-      <c r="C25" s="62" t="n"/>
-      <c r="D25" s="62" t="n"/>
-      <c r="E25" s="61" t="n"/>
+      <c r="C25" s="72" t="n"/>
+      <c r="D25" s="72" t="n"/>
+      <c r="E25" s="73" t="n"/>
     </row>
     <row r="26" ht="17" customHeight="1">
       <c r="B26" s="18" t="inlineStr">
@@ -1938,9 +2185,9 @@
           <t xml:space="preserve">  HISTORICAL REVENUE (for Y0 base)</t>
         </is>
       </c>
-      <c r="C27" s="62" t="n"/>
-      <c r="D27" s="62" t="n"/>
-      <c r="E27" s="61" t="n"/>
+      <c r="C27" s="72" t="n"/>
+      <c r="D27" s="72" t="n"/>
+      <c r="E27" s="73" t="n"/>
     </row>
     <row r="28" ht="17" customHeight="1">
       <c r="B28" s="18" t="inlineStr">
@@ -1949,7 +2196,7 @@
         </is>
       </c>
       <c r="C28" s="13" t="n">
-        <v>451442</v>
+        <v>416161</v>
       </c>
       <c r="D28" s="18" t="inlineStr">
         <is>
@@ -1978,9 +2225,9 @@
           <t xml:space="preserve">  INVESTMENT THESIS (free text)</t>
         </is>
       </c>
-      <c r="C31" s="62" t="n"/>
-      <c r="D31" s="62" t="n"/>
-      <c r="E31" s="61" t="n"/>
+      <c r="C31" s="72" t="n"/>
+      <c r="D31" s="72" t="n"/>
+      <c r="E31" s="73" t="n"/>
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="B32" s="9" t="inlineStr">
@@ -1988,9 +2235,9 @@
           <t>Company and thesis notes here.</t>
         </is>
       </c>
-      <c r="C32" s="62" t="n"/>
-      <c r="D32" s="62" t="n"/>
-      <c r="E32" s="61" t="n"/>
+      <c r="C32" s="72" t="n"/>
+      <c r="D32" s="72" t="n"/>
+      <c r="E32" s="73" t="n"/>
     </row>
     <row r="33" ht="15" customHeight="1">
       <c r="B33" s="9" t="inlineStr">
@@ -1998,9 +2245,9 @@
           <t>Key risks:</t>
         </is>
       </c>
-      <c r="C33" s="62" t="n"/>
-      <c r="D33" s="62" t="n"/>
-      <c r="E33" s="61" t="n"/>
+      <c r="C33" s="72" t="n"/>
+      <c r="D33" s="72" t="n"/>
+      <c r="E33" s="73" t="n"/>
     </row>
     <row r="34" ht="15" customHeight="1">
       <c r="B34" s="9" t="inlineStr">
@@ -2008,9 +2255,9 @@
           <t>Key catalysts:</t>
         </is>
       </c>
-      <c r="C34" s="62" t="n"/>
-      <c r="D34" s="62" t="n"/>
-      <c r="E34" s="61" t="n"/>
+      <c r="C34" s="72" t="n"/>
+      <c r="D34" s="72" t="n"/>
+      <c r="E34" s="73" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -2019,13 +2266,13 @@
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="B27:E27"/>
     <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B34:E34"/>
+    <mergeCell ref="B32:E32"/>
     <mergeCell ref="B15:E15"/>
     <mergeCell ref="B33:E33"/>
     <mergeCell ref="B25:E25"/>
     <mergeCell ref="B2:E2"/>
     <mergeCell ref="B20:E20"/>
-    <mergeCell ref="B32:E32"/>
+    <mergeCell ref="B34:E34"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2156,19 +2403,19 @@
           <t xml:space="preserve">  REVENUE</t>
         </is>
       </c>
-      <c r="C5" s="62" t="n"/>
-      <c r="D5" s="62" t="n"/>
-      <c r="E5" s="62" t="n"/>
-      <c r="F5" s="62" t="n"/>
-      <c r="G5" s="62" t="n"/>
-      <c r="H5" s="62" t="n"/>
-      <c r="I5" s="62" t="n"/>
-      <c r="J5" s="62" t="n"/>
-      <c r="K5" s="62" t="n"/>
-      <c r="L5" s="62" t="n"/>
-      <c r="M5" s="62" t="n"/>
-      <c r="N5" s="62" t="n"/>
-      <c r="O5" s="61" t="n"/>
+      <c r="C5" s="72" t="n"/>
+      <c r="D5" s="72" t="n"/>
+      <c r="E5" s="72" t="n"/>
+      <c r="F5" s="72" t="n"/>
+      <c r="G5" s="72" t="n"/>
+      <c r="H5" s="72" t="n"/>
+      <c r="I5" s="72" t="n"/>
+      <c r="J5" s="72" t="n"/>
+      <c r="K5" s="72" t="n"/>
+      <c r="L5" s="72" t="n"/>
+      <c r="M5" s="72" t="n"/>
+      <c r="N5" s="72" t="n"/>
+      <c r="O5" s="73" t="n"/>
     </row>
     <row r="6" ht="14" customHeight="1">
       <c r="B6" s="19" t="inlineStr">
@@ -2295,19 +2542,19 @@
           <t xml:space="preserve">  GROSS PROFIT</t>
         </is>
       </c>
-      <c r="C8" s="62" t="n"/>
-      <c r="D8" s="62" t="n"/>
-      <c r="E8" s="62" t="n"/>
-      <c r="F8" s="62" t="n"/>
-      <c r="G8" s="62" t="n"/>
-      <c r="H8" s="62" t="n"/>
-      <c r="I8" s="62" t="n"/>
-      <c r="J8" s="62" t="n"/>
-      <c r="K8" s="62" t="n"/>
-      <c r="L8" s="62" t="n"/>
-      <c r="M8" s="62" t="n"/>
-      <c r="N8" s="62" t="n"/>
-      <c r="O8" s="61" t="n"/>
+      <c r="C8" s="72" t="n"/>
+      <c r="D8" s="72" t="n"/>
+      <c r="E8" s="72" t="n"/>
+      <c r="F8" s="72" t="n"/>
+      <c r="G8" s="72" t="n"/>
+      <c r="H8" s="72" t="n"/>
+      <c r="I8" s="72" t="n"/>
+      <c r="J8" s="72" t="n"/>
+      <c r="K8" s="72" t="n"/>
+      <c r="L8" s="72" t="n"/>
+      <c r="M8" s="72" t="n"/>
+      <c r="N8" s="72" t="n"/>
+      <c r="O8" s="73" t="n"/>
     </row>
     <row r="9" ht="14" customHeight="1">
       <c r="B9" s="19" t="inlineStr">
@@ -2430,19 +2677,19 @@
           <t xml:space="preserve">  OPERATING EXPENSES -&gt; EBITDA</t>
         </is>
       </c>
-      <c r="C11" s="62" t="n"/>
-      <c r="D11" s="62" t="n"/>
-      <c r="E11" s="62" t="n"/>
-      <c r="F11" s="62" t="n"/>
-      <c r="G11" s="62" t="n"/>
-      <c r="H11" s="62" t="n"/>
-      <c r="I11" s="62" t="n"/>
-      <c r="J11" s="62" t="n"/>
-      <c r="K11" s="62" t="n"/>
-      <c r="L11" s="62" t="n"/>
-      <c r="M11" s="62" t="n"/>
-      <c r="N11" s="62" t="n"/>
-      <c r="O11" s="61" t="n"/>
+      <c r="C11" s="72" t="n"/>
+      <c r="D11" s="72" t="n"/>
+      <c r="E11" s="72" t="n"/>
+      <c r="F11" s="72" t="n"/>
+      <c r="G11" s="72" t="n"/>
+      <c r="H11" s="72" t="n"/>
+      <c r="I11" s="72" t="n"/>
+      <c r="J11" s="72" t="n"/>
+      <c r="K11" s="72" t="n"/>
+      <c r="L11" s="72" t="n"/>
+      <c r="M11" s="72" t="n"/>
+      <c r="N11" s="72" t="n"/>
+      <c r="O11" s="73" t="n"/>
     </row>
     <row r="12" ht="14" customHeight="1">
       <c r="B12" s="19" t="inlineStr">
@@ -2624,19 +2871,19 @@
           <t xml:space="preserve">  D&amp;A  -&gt;  EBIT</t>
         </is>
       </c>
-      <c r="C15" s="62" t="n"/>
-      <c r="D15" s="62" t="n"/>
-      <c r="E15" s="62" t="n"/>
-      <c r="F15" s="62" t="n"/>
-      <c r="G15" s="62" t="n"/>
-      <c r="H15" s="62" t="n"/>
-      <c r="I15" s="62" t="n"/>
-      <c r="J15" s="62" t="n"/>
-      <c r="K15" s="62" t="n"/>
-      <c r="L15" s="62" t="n"/>
-      <c r="M15" s="62" t="n"/>
-      <c r="N15" s="62" t="n"/>
-      <c r="O15" s="61" t="n"/>
+      <c r="C15" s="72" t="n"/>
+      <c r="D15" s="72" t="n"/>
+      <c r="E15" s="72" t="n"/>
+      <c r="F15" s="72" t="n"/>
+      <c r="G15" s="72" t="n"/>
+      <c r="H15" s="72" t="n"/>
+      <c r="I15" s="72" t="n"/>
+      <c r="J15" s="72" t="n"/>
+      <c r="K15" s="72" t="n"/>
+      <c r="L15" s="72" t="n"/>
+      <c r="M15" s="72" t="n"/>
+      <c r="N15" s="72" t="n"/>
+      <c r="O15" s="73" t="n"/>
     </row>
     <row r="16" ht="14" customHeight="1">
       <c r="B16" s="19" t="inlineStr">
@@ -2877,19 +3124,19 @@
           <t xml:space="preserve">  NOPAT  (Net Operating Profit After Tax)</t>
         </is>
       </c>
-      <c r="C20" s="62" t="n"/>
-      <c r="D20" s="62" t="n"/>
-      <c r="E20" s="62" t="n"/>
-      <c r="F20" s="62" t="n"/>
-      <c r="G20" s="62" t="n"/>
-      <c r="H20" s="62" t="n"/>
-      <c r="I20" s="62" t="n"/>
-      <c r="J20" s="62" t="n"/>
-      <c r="K20" s="62" t="n"/>
-      <c r="L20" s="62" t="n"/>
-      <c r="M20" s="62" t="n"/>
-      <c r="N20" s="62" t="n"/>
-      <c r="O20" s="61" t="n"/>
+      <c r="C20" s="72" t="n"/>
+      <c r="D20" s="72" t="n"/>
+      <c r="E20" s="72" t="n"/>
+      <c r="F20" s="72" t="n"/>
+      <c r="G20" s="72" t="n"/>
+      <c r="H20" s="72" t="n"/>
+      <c r="I20" s="72" t="n"/>
+      <c r="J20" s="72" t="n"/>
+      <c r="K20" s="72" t="n"/>
+      <c r="L20" s="72" t="n"/>
+      <c r="M20" s="72" t="n"/>
+      <c r="N20" s="72" t="n"/>
+      <c r="O20" s="73" t="n"/>
     </row>
     <row r="21" ht="14" customHeight="1">
       <c r="B21" s="19" t="inlineStr">
@@ -3012,19 +3259,19 @@
           <t xml:space="preserve">  FREE CASH FLOW TO FIRM (FCFF)</t>
         </is>
       </c>
-      <c r="C23" s="62" t="n"/>
-      <c r="D23" s="62" t="n"/>
-      <c r="E23" s="62" t="n"/>
-      <c r="F23" s="62" t="n"/>
-      <c r="G23" s="62" t="n"/>
-      <c r="H23" s="62" t="n"/>
-      <c r="I23" s="62" t="n"/>
-      <c r="J23" s="62" t="n"/>
-      <c r="K23" s="62" t="n"/>
-      <c r="L23" s="62" t="n"/>
-      <c r="M23" s="62" t="n"/>
-      <c r="N23" s="62" t="n"/>
-      <c r="O23" s="61" t="n"/>
+      <c r="C23" s="72" t="n"/>
+      <c r="D23" s="72" t="n"/>
+      <c r="E23" s="72" t="n"/>
+      <c r="F23" s="72" t="n"/>
+      <c r="G23" s="72" t="n"/>
+      <c r="H23" s="72" t="n"/>
+      <c r="I23" s="72" t="n"/>
+      <c r="J23" s="72" t="n"/>
+      <c r="K23" s="72" t="n"/>
+      <c r="L23" s="72" t="n"/>
+      <c r="M23" s="72" t="n"/>
+      <c r="N23" s="72" t="n"/>
+      <c r="O23" s="73" t="n"/>
     </row>
     <row r="24" ht="14" customHeight="1">
       <c r="B24" s="19" t="inlineStr">
@@ -3438,19 +3685,19 @@
           <t xml:space="preserve">  10-YEAR FCF PROJECTION (from model above)</t>
         </is>
       </c>
-      <c r="C32" s="62" t="n"/>
-      <c r="D32" s="62" t="n"/>
-      <c r="E32" s="62" t="n"/>
-      <c r="F32" s="62" t="n"/>
-      <c r="G32" s="62" t="n"/>
-      <c r="H32" s="62" t="n"/>
-      <c r="I32" s="62" t="n"/>
-      <c r="J32" s="62" t="n"/>
-      <c r="K32" s="62" t="n"/>
-      <c r="L32" s="62" t="n"/>
-      <c r="M32" s="62" t="n"/>
-      <c r="N32" s="62" t="n"/>
-      <c r="O32" s="61" t="n"/>
+      <c r="C32" s="72" t="n"/>
+      <c r="D32" s="72" t="n"/>
+      <c r="E32" s="72" t="n"/>
+      <c r="F32" s="72" t="n"/>
+      <c r="G32" s="72" t="n"/>
+      <c r="H32" s="72" t="n"/>
+      <c r="I32" s="72" t="n"/>
+      <c r="J32" s="72" t="n"/>
+      <c r="K32" s="72" t="n"/>
+      <c r="L32" s="72" t="n"/>
+      <c r="M32" s="72" t="n"/>
+      <c r="N32" s="72" t="n"/>
+      <c r="O32" s="73" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -3507,9 +3754,9 @@
           <t xml:space="preserve">  COST OF EQUITY  -  CAPM:  Ke = Rf + beta x ERP</t>
         </is>
       </c>
-      <c r="C4" s="62" t="n"/>
-      <c r="D4" s="62" t="n"/>
-      <c r="E4" s="61" t="n"/>
+      <c r="C4" s="72" t="n"/>
+      <c r="D4" s="72" t="n"/>
+      <c r="E4" s="73" t="n"/>
     </row>
     <row r="5" ht="17" customHeight="1">
       <c r="B5" s="18" t="inlineStr">
@@ -3548,8 +3795,8 @@
           <t xml:space="preserve">  COST OF EQUITY (Ke)</t>
         </is>
       </c>
-      <c r="C7" s="62" t="n"/>
-      <c r="D7" s="61" t="n"/>
+      <c r="C7" s="72" t="n"/>
+      <c r="D7" s="73" t="n"/>
       <c r="E7" s="40">
         <f>Assumptions!C21+Assumptions!C22*Assumptions!E21</f>
         <v/>
@@ -3561,9 +3808,9 @@
           <t xml:space="preserve">  COST OF DEBT  -  After Tax:  Kd_at = Kd x (1 - Tax Rate)</t>
         </is>
       </c>
-      <c r="C8" s="62" t="n"/>
-      <c r="D8" s="62" t="n"/>
-      <c r="E8" s="61" t="n"/>
+      <c r="C8" s="72" t="n"/>
+      <c r="D8" s="72" t="n"/>
+      <c r="E8" s="73" t="n"/>
     </row>
     <row r="9" ht="17" customHeight="1">
       <c r="B9" s="18" t="inlineStr">
@@ -3591,8 +3838,8 @@
           <t xml:space="preserve">  AFTER-TAX COST OF DEBT (Kd)</t>
         </is>
       </c>
-      <c r="C10" s="62" t="n"/>
-      <c r="D10" s="61" t="n"/>
+      <c r="C10" s="72" t="n"/>
+      <c r="D10" s="73" t="n"/>
       <c r="E10" s="40">
         <f>C9*(1-E9)</f>
         <v/>
@@ -3604,9 +3851,9 @@
           <t xml:space="preserve">  CAPITAL STRUCTURE WEIGHTS</t>
         </is>
       </c>
-      <c r="C11" s="62" t="n"/>
-      <c r="D11" s="62" t="n"/>
-      <c r="E11" s="61" t="n"/>
+      <c r="C11" s="72" t="n"/>
+      <c r="D11" s="72" t="n"/>
+      <c r="E11" s="73" t="n"/>
     </row>
     <row r="12" ht="17" customHeight="1">
       <c r="B12" s="18" t="inlineStr">
@@ -3654,9 +3901,9 @@
           <t xml:space="preserve">  WACC CALCULATION</t>
         </is>
       </c>
-      <c r="C14" s="62" t="n"/>
-      <c r="D14" s="62" t="n"/>
-      <c r="E14" s="61" t="n"/>
+      <c r="C14" s="72" t="n"/>
+      <c r="D14" s="72" t="n"/>
+      <c r="E14" s="73" t="n"/>
     </row>
     <row r="15" ht="17" customHeight="1">
       <c r="B15" s="18" t="inlineStr">
@@ -3684,8 +3931,8 @@
           <t xml:space="preserve">  WACC  =  Ke x We  +  Kd(1-t) x Wd</t>
         </is>
       </c>
-      <c r="C16" s="62" t="n"/>
-      <c r="D16" s="61" t="n"/>
+      <c r="C16" s="72" t="n"/>
+      <c r="D16" s="73" t="n"/>
       <c r="E16" s="43">
         <f>C15+E15</f>
         <v/>
@@ -3750,9 +3997,9 @@
           <t xml:space="preserve">  DISCOUNT RATE &amp; KEY INPUTS</t>
         </is>
       </c>
-      <c r="C3" s="62" t="n"/>
-      <c r="D3" s="62" t="n"/>
-      <c r="E3" s="61" t="n"/>
+      <c r="C3" s="72" t="n"/>
+      <c r="D3" s="72" t="n"/>
+      <c r="E3" s="73" t="n"/>
     </row>
     <row r="4" ht="17" customHeight="1">
       <c r="B4" s="18" t="inlineStr">
@@ -3764,8 +4011,12 @@
         <f>WACC!E16</f>
         <v/>
       </c>
-      <c r="D4" s="22" t="inlineStr"/>
-      <c r="E4" s="22" t="inlineStr"/>
+      <c r="D4" s="45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Ke×We + Kd(1-t)×Wd  —  from WACC sheet</t>
+        </is>
+      </c>
+      <c r="E4" s="73" t="n"/>
     </row>
     <row r="5" ht="17" customHeight="1">
       <c r="B5" s="18" t="inlineStr">
@@ -3777,8 +4028,12 @@
         <f>Assumptions!C26</f>
         <v/>
       </c>
-      <c r="D5" s="22" t="inlineStr"/>
-      <c r="E5" s="22" t="inlineStr"/>
+      <c r="D5" s="45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Long-run FCF growth after Year 10  —  Assumptions</t>
+        </is>
+      </c>
+      <c r="E5" s="73" t="n"/>
     </row>
     <row r="6" ht="17" customHeight="1">
       <c r="B6" s="18" t="inlineStr">
@@ -3786,12 +4041,16 @@
           <t xml:space="preserve">  Exit EBITDA Multiple</t>
         </is>
       </c>
-      <c r="C6" s="45">
+      <c r="C6" s="46">
         <f>Assumptions!E26</f>
         <v/>
       </c>
-      <c r="D6" s="22" t="inlineStr"/>
-      <c r="E6" s="22" t="inlineStr"/>
+      <c r="D6" s="45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Reference only; Gordon Growth is primary TV method</t>
+        </is>
+      </c>
+      <c r="E6" s="73" t="n"/>
     </row>
     <row r="7" ht="17" customHeight="1">
       <c r="B7" s="18" t="inlineStr">
@@ -3803,8 +4062,12 @@
         <f>Assumptions!C8-Assumptions!E8</f>
         <v/>
       </c>
-      <c r="D7" s="22" t="inlineStr"/>
-      <c r="E7" s="22" t="inlineStr"/>
+      <c r="D7" s="45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Total Debt minus Cash  —  from Assumptions</t>
+        </is>
+      </c>
+      <c r="E7" s="73" t="n"/>
     </row>
     <row r="8" ht="17" customHeight="1">
       <c r="B8" s="18" t="inlineStr">
@@ -3816,8 +4079,12 @@
         <f>Assumptions!E7</f>
         <v/>
       </c>
-      <c r="D8" s="22" t="inlineStr"/>
-      <c r="E8" s="22" t="inlineStr"/>
+      <c r="D8" s="45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Diluted share count  —  from Assumptions</t>
+        </is>
+      </c>
+      <c r="E8" s="73" t="n"/>
     </row>
     <row r="9" ht="16" customHeight="1">
       <c r="B9" s="11" t="inlineStr">
@@ -3825,9 +4092,9 @@
           <t xml:space="preserve">  PROJECTED FCF BY YEAR  (from Income Statement)</t>
         </is>
       </c>
-      <c r="C9" s="62" t="n"/>
-      <c r="D9" s="62" t="n"/>
-      <c r="E9" s="61" t="n"/>
+      <c r="C9" s="72" t="n"/>
+      <c r="D9" s="72" t="n"/>
+      <c r="E9" s="73" t="n"/>
     </row>
     <row r="10" ht="14" customHeight="1">
       <c r="B10" s="18" t="inlineStr">
@@ -3835,52 +4102,52 @@
           <t xml:space="preserve">  Year</t>
         </is>
       </c>
-      <c r="C10" s="46" t="inlineStr">
+      <c r="C10" s="47" t="inlineStr">
         <is>
           <t>FY2027</t>
         </is>
       </c>
-      <c r="D10" s="46" t="inlineStr">
+      <c r="D10" s="47" t="inlineStr">
         <is>
           <t>FY2028</t>
         </is>
       </c>
-      <c r="E10" s="46" t="inlineStr">
+      <c r="E10" s="47" t="inlineStr">
         <is>
           <t>FY2029</t>
         </is>
       </c>
-      <c r="F10" s="46" t="inlineStr">
+      <c r="F10" s="47" t="inlineStr">
         <is>
           <t>FY2030</t>
         </is>
       </c>
-      <c r="G10" s="46" t="inlineStr">
+      <c r="G10" s="47" t="inlineStr">
         <is>
           <t>FY2031</t>
         </is>
       </c>
-      <c r="H10" s="46" t="inlineStr">
+      <c r="H10" s="47" t="inlineStr">
         <is>
           <t>FY2032</t>
         </is>
       </c>
-      <c r="I10" s="46" t="inlineStr">
+      <c r="I10" s="47" t="inlineStr">
         <is>
           <t>FY2033</t>
         </is>
       </c>
-      <c r="J10" s="46" t="inlineStr">
+      <c r="J10" s="47" t="inlineStr">
         <is>
           <t>FY2034</t>
         </is>
       </c>
-      <c r="K10" s="46" t="inlineStr">
+      <c r="K10" s="47" t="inlineStr">
         <is>
           <t>FY2035</t>
         </is>
       </c>
-      <c r="L10" s="46" t="inlineStr">
+      <c r="L10" s="47" t="inlineStr">
         <is>
           <t>FY2036</t>
         </is>
@@ -3939,34 +4206,34 @@
           <t xml:space="preserve">  Discount Period (t)</t>
         </is>
       </c>
-      <c r="C12" s="45" t="n">
+      <c r="C12" s="46" t="n">
         <v>1</v>
       </c>
-      <c r="D12" s="45" t="n">
+      <c r="D12" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="E12" s="45" t="n">
+      <c r="E12" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="F12" s="45" t="n">
+      <c r="F12" s="46" t="n">
         <v>4</v>
       </c>
-      <c r="G12" s="45" t="n">
+      <c r="G12" s="46" t="n">
         <v>5</v>
       </c>
-      <c r="H12" s="45" t="n">
+      <c r="H12" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="I12" s="45" t="n">
+      <c r="I12" s="46" t="n">
         <v>7</v>
       </c>
-      <c r="J12" s="45" t="n">
+      <c r="J12" s="46" t="n">
         <v>8</v>
       </c>
-      <c r="K12" s="45" t="n">
+      <c r="K12" s="46" t="n">
         <v>9</v>
       </c>
-      <c r="L12" s="45" t="n">
+      <c r="L12" s="46" t="n">
         <v>10</v>
       </c>
     </row>
@@ -3976,43 +4243,43 @@
           <t xml:space="preserve">  Discount Factor  [1/(1+WACC)^t]</t>
         </is>
       </c>
-      <c r="C13" s="47">
+      <c r="C13" s="48">
         <f>1/(1+C4)^C12</f>
         <v/>
       </c>
-      <c r="D13" s="47">
+      <c r="D13" s="48">
         <f>1/(1+C4)^D12</f>
         <v/>
       </c>
-      <c r="E13" s="47">
+      <c r="E13" s="48">
         <f>1/(1+C4)^E12</f>
         <v/>
       </c>
-      <c r="F13" s="47">
+      <c r="F13" s="48">
         <f>1/(1+C4)^F12</f>
         <v/>
       </c>
-      <c r="G13" s="47">
+      <c r="G13" s="48">
         <f>1/(1+C4)^G12</f>
         <v/>
       </c>
-      <c r="H13" s="47">
+      <c r="H13" s="48">
         <f>1/(1+C4)^H12</f>
         <v/>
       </c>
-      <c r="I13" s="47">
+      <c r="I13" s="48">
         <f>1/(1+C4)^I12</f>
         <v/>
       </c>
-      <c r="J13" s="47">
+      <c r="J13" s="48">
         <f>1/(1+C4)^J12</f>
         <v/>
       </c>
-      <c r="K13" s="47">
+      <c r="K13" s="48">
         <f>1/(1+C4)^K12</f>
         <v/>
       </c>
-      <c r="L13" s="47">
+      <c r="L13" s="48">
         <f>1/(1+C4)^L12</f>
         <v/>
       </c>
@@ -4081,9 +4348,9 @@
           <t xml:space="preserve">  TERMINAL VALUE</t>
         </is>
       </c>
-      <c r="C16" s="62" t="n"/>
-      <c r="D16" s="62" t="n"/>
-      <c r="E16" s="61" t="n"/>
+      <c r="C16" s="72" t="n"/>
+      <c r="D16" s="72" t="n"/>
+      <c r="E16" s="73" t="n"/>
     </row>
     <row r="17" ht="17" customHeight="1">
       <c r="B17" s="18" t="inlineStr">
@@ -4131,9 +4398,9 @@
           <t xml:space="preserve">  VALUATION BRIDGE</t>
         </is>
       </c>
-      <c r="C19" s="62" t="n"/>
-      <c r="D19" s="62" t="n"/>
-      <c r="E19" s="61" t="n"/>
+      <c r="C19" s="72" t="n"/>
+      <c r="D19" s="72" t="n"/>
+      <c r="E19" s="73" t="n"/>
     </row>
     <row r="20" ht="17" customHeight="1">
       <c r="B20" s="18" t="inlineStr">
@@ -4158,12 +4425,12 @@
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="B22" s="48" t="inlineStr">
+      <c r="B22" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  ENTERPRISE VALUE</t>
         </is>
       </c>
-      <c r="C22" s="49">
+      <c r="C22" s="50">
         <f>C20+C21</f>
         <v/>
       </c>
@@ -4180,12 +4447,12 @@
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
-      <c r="B24" s="48" t="inlineStr">
+      <c r="B24" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  EQUITY VALUE</t>
         </is>
       </c>
-      <c r="C24" s="49">
+      <c r="C24" s="50">
         <f>C22-C23</f>
         <v/>
       </c>
@@ -4202,12 +4469,12 @@
       </c>
     </row>
     <row r="26" ht="28" customHeight="1">
-      <c r="B26" s="50" t="inlineStr">
+      <c r="B26" s="51" t="inlineStr">
         <is>
           <t xml:space="preserve">  IMPLIED SHARE PRICE (DCF)</t>
         </is>
       </c>
-      <c r="C26" s="51">
+      <c r="C26" s="52">
         <f>C24/C25</f>
         <v/>
       </c>
@@ -4218,7 +4485,7 @@
           <t xml:space="preserve">  Current Stock Price ($)</t>
         </is>
       </c>
-      <c r="C27" s="52">
+      <c r="C27" s="53">
         <f>Assumptions!C7</f>
         <v/>
       </c>
@@ -4229,7 +4496,7 @@
           <t xml:space="preserve">  Upside / (Downside) %</t>
         </is>
       </c>
-      <c r="C28" s="53">
+      <c r="C28" s="54">
         <f>(C26-C27)/C27</f>
         <v/>
       </c>
@@ -4240,9 +4507,9 @@
           <t xml:space="preserve">  VALUATION COMPOSITION</t>
         </is>
       </c>
-      <c r="C29" s="62" t="n"/>
-      <c r="D29" s="62" t="n"/>
-      <c r="E29" s="61" t="n"/>
+      <c r="C29" s="72" t="n"/>
+      <c r="D29" s="72" t="n"/>
+      <c r="E29" s="73" t="n"/>
     </row>
     <row r="30" ht="17" customHeight="1">
       <c r="B30" s="18" t="inlineStr">
@@ -4250,7 +4517,7 @@
           <t xml:space="preserve">  PV of FCFs as % of Enterprise Value</t>
         </is>
       </c>
-      <c r="C30" s="54">
+      <c r="C30" s="55">
         <f>IF(C22=0,0,C20/C22)</f>
         <v/>
       </c>
@@ -4261,7 +4528,7 @@
           <t xml:space="preserve">  PV of Terminal Value as % of Enterprise Value</t>
         </is>
       </c>
-      <c r="C31" s="54">
+      <c r="C31" s="55">
         <f>IF(C22=0,0,C21/C22)</f>
         <v/>
       </c>
@@ -4272,17 +4539,22 @@
           <t xml:space="preserve">  Implied EV / EBITDA Multiple (LTM)</t>
         </is>
       </c>
-      <c r="C32" s="45">
+      <c r="C32" s="46">
         <f>IF('Income Statement'!E13=0,0,C22/'Income Statement'!E13)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="11">
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="D6:E6"/>
     <mergeCell ref="B9:E9"/>
     <mergeCell ref="B1:E1"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="D5:E5"/>
     <mergeCell ref="B16:E16"/>
     <mergeCell ref="B29:E29"/>
+    <mergeCell ref="D4:E4"/>
     <mergeCell ref="B3:E3"/>
     <mergeCell ref="B19:E19"/>
   </mergeCells>
@@ -4326,494 +4598,494 @@
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">
-      <c r="B4" s="55" t="inlineStr">
+      <c r="B4" s="56" t="inlineStr">
         <is>
           <t xml:space="preserve">  TABLE 1 - Implied Share Price  vs  WACC  x  Terminal Growth Rate</t>
         </is>
       </c>
-      <c r="C4" s="62" t="n"/>
-      <c r="D4" s="62" t="n"/>
-      <c r="E4" s="62" t="n"/>
-      <c r="F4" s="62" t="n"/>
-      <c r="G4" s="62" t="n"/>
-      <c r="H4" s="62" t="n"/>
-      <c r="I4" s="61" t="n"/>
+      <c r="C4" s="72" t="n"/>
+      <c r="D4" s="72" t="n"/>
+      <c r="E4" s="72" t="n"/>
+      <c r="F4" s="72" t="n"/>
+      <c r="G4" s="72" t="n"/>
+      <c r="H4" s="72" t="n"/>
+      <c r="I4" s="73" t="n"/>
     </row>
     <row r="5" ht="16" customHeight="1">
-      <c r="B5" s="56" t="inlineStr">
+      <c r="B5" s="57" t="inlineStr">
         <is>
           <t xml:space="preserve">  WACC \ TGR</t>
         </is>
       </c>
-      <c r="C5" s="57">
+      <c r="C5" s="58">
         <f>'DCF Valuation'!C5+(-0.01)</f>
         <v/>
       </c>
-      <c r="D5" s="57">
+      <c r="D5" s="58">
         <f>'DCF Valuation'!C5+(-0.005)</f>
         <v/>
       </c>
-      <c r="E5" s="57">
+      <c r="E5" s="58">
         <f>'DCF Valuation'!C5+(0.0)</f>
         <v/>
       </c>
-      <c r="F5" s="57">
+      <c r="F5" s="58">
         <f>'DCF Valuation'!C5+(0.005)</f>
         <v/>
       </c>
-      <c r="G5" s="57">
+      <c r="G5" s="58">
         <f>'DCF Valuation'!C5+(0.01)</f>
         <v/>
       </c>
-      <c r="H5" s="57">
+      <c r="H5" s="58">
         <f>'DCF Valuation'!C5+(0.015)</f>
         <v/>
       </c>
     </row>
     <row r="6" ht="17" customHeight="1">
-      <c r="B6" s="58">
+      <c r="B6" s="59">
         <f>'DCF Valuation'!C4+(-0.015)</f>
         <v/>
       </c>
-      <c r="C6" s="52">
+      <c r="C6" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B6)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+C5)/MAX(B6-C5,0.0001)/(1+B6)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
-      <c r="D6" s="52">
+      <c r="D6" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B6)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+D5)/MAX(B6-D5,0.0001)/(1+B6)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
-      <c r="E6" s="52">
+      <c r="E6" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B6)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+E5)/MAX(B6-E5,0.0001)/(1+B6)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
-      <c r="F6" s="52">
+      <c r="F6" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B6)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+F5)/MAX(B6-F5,0.0001)/(1+B6)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
-      <c r="G6" s="52">
+      <c r="G6" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B6)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+G5)/MAX(B6-G5,0.0001)/(1+B6)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
-      <c r="H6" s="52">
+      <c r="H6" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B6)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+H5)/MAX(B6-H5,0.0001)/(1+B6)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
     </row>
     <row r="7" ht="17" customHeight="1">
-      <c r="B7" s="58">
+      <c r="B7" s="59">
         <f>'DCF Valuation'!C4+(-0.01)</f>
         <v/>
       </c>
-      <c r="C7" s="52">
+      <c r="C7" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B7)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+C5)/MAX(B7-C5,0.0001)/(1+B7)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
-      <c r="D7" s="52">
+      <c r="D7" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B7)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+D5)/MAX(B7-D5,0.0001)/(1+B7)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
-      <c r="E7" s="52">
+      <c r="E7" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B7)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+E5)/MAX(B7-E5,0.0001)/(1+B7)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
-      <c r="F7" s="52">
+      <c r="F7" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B7)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+F5)/MAX(B7-F5,0.0001)/(1+B7)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
-      <c r="G7" s="52">
+      <c r="G7" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B7)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+G5)/MAX(B7-G5,0.0001)/(1+B7)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
-      <c r="H7" s="52">
+      <c r="H7" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B7)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+H5)/MAX(B7-H5,0.0001)/(1+B7)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="17" customHeight="1">
-      <c r="B8" s="58">
+      <c r="B8" s="59">
         <f>'DCF Valuation'!C4+(-0.005)</f>
         <v/>
       </c>
-      <c r="C8" s="52">
+      <c r="C8" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B8)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+C5)/MAX(B8-C5,0.0001)/(1+B8)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
-      <c r="D8" s="52">
+      <c r="D8" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B8)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+D5)/MAX(B8-D5,0.0001)/(1+B8)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
-      <c r="E8" s="52">
+      <c r="E8" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B8)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+E5)/MAX(B8-E5,0.0001)/(1+B8)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
-      <c r="F8" s="52">
+      <c r="F8" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B8)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+F5)/MAX(B8-F5,0.0001)/(1+B8)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
-      <c r="G8" s="52">
+      <c r="G8" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B8)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+G5)/MAX(B8-G5,0.0001)/(1+B8)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
-      <c r="H8" s="52">
+      <c r="H8" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B8)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+H5)/MAX(B8-H5,0.0001)/(1+B8)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="17" customHeight="1">
-      <c r="B9" s="58">
+      <c r="B9" s="59">
         <f>'DCF Valuation'!C4+(0.0)</f>
         <v/>
       </c>
-      <c r="C9" s="52">
+      <c r="C9" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B9)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+C5)/MAX(B9-C5,0.0001)/(1+B9)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
-      <c r="D9" s="52">
+      <c r="D9" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B9)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+D5)/MAX(B9-D5,0.0001)/(1+B9)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
-      <c r="E9" s="52">
+      <c r="E9" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B9)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+E5)/MAX(B9-E5,0.0001)/(1+B9)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
-      <c r="F9" s="52">
+      <c r="F9" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B9)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+F5)/MAX(B9-F5,0.0001)/(1+B9)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
-      <c r="G9" s="52">
+      <c r="G9" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B9)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+G5)/MAX(B9-G5,0.0001)/(1+B9)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
-      <c r="H9" s="52">
+      <c r="H9" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B9)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+H5)/MAX(B9-H5,0.0001)/(1+B9)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="17" customHeight="1">
-      <c r="B10" s="58">
+      <c r="B10" s="59">
         <f>'DCF Valuation'!C4+(0.005)</f>
         <v/>
       </c>
-      <c r="C10" s="52">
+      <c r="C10" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B10)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+C5)/MAX(B10-C5,0.0001)/(1+B10)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
-      <c r="D10" s="52">
+      <c r="D10" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B10)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+D5)/MAX(B10-D5,0.0001)/(1+B10)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
-      <c r="E10" s="52">
+      <c r="E10" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B10)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+E5)/MAX(B10-E5,0.0001)/(1+B10)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
-      <c r="F10" s="52">
+      <c r="F10" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B10)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+F5)/MAX(B10-F5,0.0001)/(1+B10)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
-      <c r="G10" s="52">
+      <c r="G10" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B10)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+G5)/MAX(B10-G5,0.0001)/(1+B10)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
-      <c r="H10" s="52">
+      <c r="H10" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B10)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+H5)/MAX(B10-H5,0.0001)/(1+B10)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="17" customHeight="1">
-      <c r="B11" s="58">
+      <c r="B11" s="59">
         <f>'DCF Valuation'!C4+(0.01)</f>
         <v/>
       </c>
-      <c r="C11" s="52">
+      <c r="C11" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B11)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+C5)/MAX(B11-C5,0.0001)/(1+B11)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
-      <c r="D11" s="52">
+      <c r="D11" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B11)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+D5)/MAX(B11-D5,0.0001)/(1+B11)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
-      <c r="E11" s="52">
+      <c r="E11" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B11)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+E5)/MAX(B11-E5,0.0001)/(1+B11)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
-      <c r="F11" s="52">
+      <c r="F11" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B11)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+F5)/MAX(B11-F5,0.0001)/(1+B11)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
-      <c r="G11" s="52">
+      <c r="G11" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B11)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+G5)/MAX(B11-G5,0.0001)/(1+B11)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
-      <c r="H11" s="52">
+      <c r="H11" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B11)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+H5)/MAX(B11-H5,0.0001)/(1+B11)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
     </row>
     <row r="12" ht="17" customHeight="1">
-      <c r="B12" s="58">
+      <c r="B12" s="59">
         <f>'DCF Valuation'!C4+(0.015)</f>
         <v/>
       </c>
-      <c r="C12" s="52">
+      <c r="C12" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B12)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+C5)/MAX(B12-C5,0.0001)/(1+B12)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
-      <c r="D12" s="52">
+      <c r="D12" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B12)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+D5)/MAX(B12-D5,0.0001)/(1+B12)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
-      <c r="E12" s="52">
+      <c r="E12" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B12)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+E5)/MAX(B12-E5,0.0001)/(1+B12)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
-      <c r="F12" s="52">
+      <c r="F12" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B12)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+F5)/MAX(B12-F5,0.0001)/(1+B12)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
-      <c r="G12" s="52">
+      <c r="G12" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B12)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+G5)/MAX(B12-G5,0.0001)/(1+B12)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
-      <c r="H12" s="52">
+      <c r="H12" s="53">
         <f>IFERROR((SUMPRODUCT('Income Statement'!F29:O29,1/(1+B12)^{1,2,3,4,5,6,7,8,9,10})+'Income Statement'!O29*(1+H5)/MAX(B12-H5,0.0001)/(1+B12)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"—")</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="16" customHeight="1">
-      <c r="B14" s="55" t="inlineStr">
+      <c r="B14" s="56" t="inlineStr">
         <is>
           <t xml:space="preserve">  TABLE 2 - Implied Share Price  vs  EBITDA Margin  x  Y1 Revenue Growth</t>
         </is>
       </c>
-      <c r="C14" s="62" t="n"/>
-      <c r="D14" s="62" t="n"/>
-      <c r="E14" s="62" t="n"/>
-      <c r="F14" s="62" t="n"/>
-      <c r="G14" s="62" t="n"/>
-      <c r="H14" s="61" t="n"/>
+      <c r="C14" s="72" t="n"/>
+      <c r="D14" s="72" t="n"/>
+      <c r="E14" s="72" t="n"/>
+      <c r="F14" s="72" t="n"/>
+      <c r="G14" s="72" t="n"/>
+      <c r="H14" s="73" t="n"/>
     </row>
     <row r="15" ht="16" customHeight="1">
-      <c r="B15" s="56" t="inlineStr">
+      <c r="B15" s="57" t="inlineStr">
         <is>
           <t xml:space="preserve">  Rev Gr\EBITDA%</t>
         </is>
       </c>
-      <c r="C15" s="59">
+      <c r="C15" s="60">
         <f>Assumptions!E16+(-0.04)</f>
         <v/>
       </c>
-      <c r="D15" s="59">
+      <c r="D15" s="60">
         <f>Assumptions!E16+(-0.02)</f>
         <v/>
       </c>
-      <c r="E15" s="59">
+      <c r="E15" s="60">
         <f>Assumptions!E16+(0.0)</f>
         <v/>
       </c>
-      <c r="F15" s="59">
+      <c r="F15" s="60">
         <f>Assumptions!E16+(0.02)</f>
         <v/>
       </c>
-      <c r="G15" s="59">
+      <c r="G15" s="60">
         <f>Assumptions!E16+(0.04)</f>
         <v/>
       </c>
     </row>
     <row r="16" ht="17" customHeight="1">
-      <c r="B16" s="60">
+      <c r="B16" s="61">
         <f>Assumptions!C10+(-0.03)</f>
         <v/>
       </c>
-      <c r="C16" s="52">
+      <c r="C16" s="53">
         <f>IFERROR('DCF Valuation'!C26*((1+B16)/(1+Assumptions!C10))*(C15/Assumptions!E16),"—")</f>
         <v/>
       </c>
-      <c r="D16" s="52">
+      <c r="D16" s="53">
         <f>IFERROR('DCF Valuation'!C26*((1+B16)/(1+Assumptions!C10))*(D15/Assumptions!E16),"—")</f>
         <v/>
       </c>
-      <c r="E16" s="52">
+      <c r="E16" s="53">
         <f>IFERROR('DCF Valuation'!C26*((1+B16)/(1+Assumptions!C10))*(E15/Assumptions!E16),"—")</f>
         <v/>
       </c>
-      <c r="F16" s="52">
+      <c r="F16" s="53">
         <f>IFERROR('DCF Valuation'!C26*((1+B16)/(1+Assumptions!C10))*(F15/Assumptions!E16),"—")</f>
         <v/>
       </c>
-      <c r="G16" s="52">
+      <c r="G16" s="53">
         <f>IFERROR('DCF Valuation'!C26*((1+B16)/(1+Assumptions!C10))*(G15/Assumptions!E16),"—")</f>
         <v/>
       </c>
     </row>
     <row r="17" ht="17" customHeight="1">
-      <c r="B17" s="60">
+      <c r="B17" s="61">
         <f>Assumptions!C10+(-0.02)</f>
         <v/>
       </c>
-      <c r="C17" s="52">
+      <c r="C17" s="53">
         <f>IFERROR('DCF Valuation'!C26*((1+B17)/(1+Assumptions!C10))*(C15/Assumptions!E16),"—")</f>
         <v/>
       </c>
-      <c r="D17" s="52">
+      <c r="D17" s="53">
         <f>IFERROR('DCF Valuation'!C26*((1+B17)/(1+Assumptions!C10))*(D15/Assumptions!E16),"—")</f>
         <v/>
       </c>
-      <c r="E17" s="52">
+      <c r="E17" s="53">
         <f>IFERROR('DCF Valuation'!C26*((1+B17)/(1+Assumptions!C10))*(E15/Assumptions!E16),"—")</f>
         <v/>
       </c>
-      <c r="F17" s="52">
+      <c r="F17" s="53">
         <f>IFERROR('DCF Valuation'!C26*((1+B17)/(1+Assumptions!C10))*(F15/Assumptions!E16),"—")</f>
         <v/>
       </c>
-      <c r="G17" s="52">
+      <c r="G17" s="53">
         <f>IFERROR('DCF Valuation'!C26*((1+B17)/(1+Assumptions!C10))*(G15/Assumptions!E16),"—")</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="17" customHeight="1">
-      <c r="B18" s="60">
+      <c r="B18" s="61">
         <f>Assumptions!C10+(-0.01)</f>
         <v/>
       </c>
-      <c r="C18" s="52">
+      <c r="C18" s="53">
         <f>IFERROR('DCF Valuation'!C26*((1+B18)/(1+Assumptions!C10))*(C15/Assumptions!E16),"—")</f>
         <v/>
       </c>
-      <c r="D18" s="52">
+      <c r="D18" s="53">
         <f>IFERROR('DCF Valuation'!C26*((1+B18)/(1+Assumptions!C10))*(D15/Assumptions!E16),"—")</f>
         <v/>
       </c>
-      <c r="E18" s="52">
+      <c r="E18" s="53">
         <f>IFERROR('DCF Valuation'!C26*((1+B18)/(1+Assumptions!C10))*(E15/Assumptions!E16),"—")</f>
         <v/>
       </c>
-      <c r="F18" s="52">
+      <c r="F18" s="53">
         <f>IFERROR('DCF Valuation'!C26*((1+B18)/(1+Assumptions!C10))*(F15/Assumptions!E16),"—")</f>
         <v/>
       </c>
-      <c r="G18" s="52">
+      <c r="G18" s="53">
         <f>IFERROR('DCF Valuation'!C26*((1+B18)/(1+Assumptions!C10))*(G15/Assumptions!E16),"—")</f>
         <v/>
       </c>
     </row>
     <row r="19" ht="17" customHeight="1">
-      <c r="B19" s="60">
+      <c r="B19" s="61">
         <f>Assumptions!C10+(0.0)</f>
         <v/>
       </c>
-      <c r="C19" s="52">
+      <c r="C19" s="53">
         <f>IFERROR('DCF Valuation'!C26*((1+B19)/(1+Assumptions!C10))*(C15/Assumptions!E16),"—")</f>
         <v/>
       </c>
-      <c r="D19" s="52">
+      <c r="D19" s="53">
         <f>IFERROR('DCF Valuation'!C26*((1+B19)/(1+Assumptions!C10))*(D15/Assumptions!E16),"—")</f>
         <v/>
       </c>
-      <c r="E19" s="52">
+      <c r="E19" s="53">
         <f>IFERROR('DCF Valuation'!C26*((1+B19)/(1+Assumptions!C10))*(E15/Assumptions!E16),"—")</f>
         <v/>
       </c>
-      <c r="F19" s="52">
+      <c r="F19" s="53">
         <f>IFERROR('DCF Valuation'!C26*((1+B19)/(1+Assumptions!C10))*(F15/Assumptions!E16),"—")</f>
         <v/>
       </c>
-      <c r="G19" s="52">
+      <c r="G19" s="53">
         <f>IFERROR('DCF Valuation'!C26*((1+B19)/(1+Assumptions!C10))*(G15/Assumptions!E16),"—")</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="17" customHeight="1">
-      <c r="B20" s="60">
+      <c r="B20" s="61">
         <f>Assumptions!C10+(0.01)</f>
         <v/>
       </c>
-      <c r="C20" s="52">
+      <c r="C20" s="53">
         <f>IFERROR('DCF Valuation'!C26*((1+B20)/(1+Assumptions!C10))*(C15/Assumptions!E16),"—")</f>
         <v/>
       </c>
-      <c r="D20" s="52">
+      <c r="D20" s="53">
         <f>IFERROR('DCF Valuation'!C26*((1+B20)/(1+Assumptions!C10))*(D15/Assumptions!E16),"—")</f>
         <v/>
       </c>
-      <c r="E20" s="52">
+      <c r="E20" s="53">
         <f>IFERROR('DCF Valuation'!C26*((1+B20)/(1+Assumptions!C10))*(E15/Assumptions!E16),"—")</f>
         <v/>
       </c>
-      <c r="F20" s="52">
+      <c r="F20" s="53">
         <f>IFERROR('DCF Valuation'!C26*((1+B20)/(1+Assumptions!C10))*(F15/Assumptions!E16),"—")</f>
         <v/>
       </c>
-      <c r="G20" s="52">
+      <c r="G20" s="53">
         <f>IFERROR('DCF Valuation'!C26*((1+B20)/(1+Assumptions!C10))*(G15/Assumptions!E16),"—")</f>
         <v/>
       </c>
     </row>
     <row r="21" ht="17" customHeight="1">
-      <c r="B21" s="60">
+      <c r="B21" s="61">
         <f>Assumptions!C10+(0.02)</f>
         <v/>
       </c>
-      <c r="C21" s="52">
+      <c r="C21" s="53">
         <f>IFERROR('DCF Valuation'!C26*((1+B21)/(1+Assumptions!C10))*(C15/Assumptions!E16),"—")</f>
         <v/>
       </c>
-      <c r="D21" s="52">
+      <c r="D21" s="53">
         <f>IFERROR('DCF Valuation'!C26*((1+B21)/(1+Assumptions!C10))*(D15/Assumptions!E16),"—")</f>
         <v/>
       </c>
-      <c r="E21" s="52">
+      <c r="E21" s="53">
         <f>IFERROR('DCF Valuation'!C26*((1+B21)/(1+Assumptions!C10))*(E15/Assumptions!E16),"—")</f>
         <v/>
       </c>
-      <c r="F21" s="52">
+      <c r="F21" s="53">
         <f>IFERROR('DCF Valuation'!C26*((1+B21)/(1+Assumptions!C10))*(F15/Assumptions!E16),"—")</f>
         <v/>
       </c>
-      <c r="G21" s="52">
+      <c r="G21" s="53">
         <f>IFERROR('DCF Valuation'!C26*((1+B21)/(1+Assumptions!C10))*(G15/Assumptions!E16),"—")</f>
         <v/>
       </c>
     </row>
     <row r="22" ht="17" customHeight="1">
-      <c r="B22" s="60">
+      <c r="B22" s="61">
         <f>Assumptions!C10+(0.03)</f>
         <v/>
       </c>
-      <c r="C22" s="52">
+      <c r="C22" s="53">
         <f>IFERROR('DCF Valuation'!C26*((1+B22)/(1+Assumptions!C10))*(C15/Assumptions!E16),"—")</f>
         <v/>
       </c>
-      <c r="D22" s="52">
+      <c r="D22" s="53">
         <f>IFERROR('DCF Valuation'!C26*((1+B22)/(1+Assumptions!C10))*(D15/Assumptions!E16),"—")</f>
         <v/>
       </c>
-      <c r="E22" s="52">
+      <c r="E22" s="53">
         <f>IFERROR('DCF Valuation'!C26*((1+B22)/(1+Assumptions!C10))*(E15/Assumptions!E16),"—")</f>
         <v/>
       </c>
-      <c r="F22" s="52">
+      <c r="F22" s="53">
         <f>IFERROR('DCF Valuation'!C26*((1+B22)/(1+Assumptions!C10))*(F15/Assumptions!E16),"—")</f>
         <v/>
       </c>
-      <c r="G22" s="52">
+      <c r="G22" s="53">
         <f>IFERROR('DCF Valuation'!C26*((1+B22)/(1+Assumptions!C10))*(G15/Assumptions!E16),"—")</f>
         <v/>
       </c>
     </row>
     <row r="24" ht="16" customHeight="1">
-      <c r="B24" s="55" t="inlineStr">
+      <c r="B24" s="56" t="inlineStr">
         <is>
           <t xml:space="preserve">  FOOTBALL FIELD  -  Valuation Range Summary</t>
         </is>
       </c>
-      <c r="C24" s="62" t="n"/>
-      <c r="D24" s="62" t="n"/>
-      <c r="E24" s="62" t="n"/>
-      <c r="F24" s="62" t="n"/>
-      <c r="G24" s="62" t="n"/>
-      <c r="H24" s="61" t="n"/>
+      <c r="C24" s="72" t="n"/>
+      <c r="D24" s="72" t="n"/>
+      <c r="E24" s="72" t="n"/>
+      <c r="F24" s="72" t="n"/>
+      <c r="G24" s="72" t="n"/>
+      <c r="H24" s="73" t="n"/>
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="B25" s="31" t="inlineStr">
@@ -4848,15 +5120,15 @@
           <t xml:space="preserve">  DCF  (base case)</t>
         </is>
       </c>
-      <c r="C26" s="52">
+      <c r="C26" s="53">
         <f>'DCF Valuation'!C26</f>
         <v/>
       </c>
-      <c r="D26" s="52">
+      <c r="D26" s="53">
         <f>'DCF Valuation'!C26</f>
         <v/>
       </c>
-      <c r="E26" s="52">
+      <c r="E26" s="53">
         <f>Assumptions!C7</f>
         <v/>
       </c>
@@ -4872,15 +5144,15 @@
           <t xml:space="preserve">  DCF  (bull: FCF+15%)</t>
         </is>
       </c>
-      <c r="C27" s="52">
+      <c r="C27" s="53">
         <f>'DCF Valuation'!C26*1.12</f>
         <v/>
       </c>
-      <c r="D27" s="52">
+      <c r="D27" s="53">
         <f>'DCF Valuation'!C26*1.22</f>
         <v/>
       </c>
-      <c r="E27" s="52">
+      <c r="E27" s="53">
         <f>Assumptions!C7</f>
         <v/>
       </c>
@@ -4896,15 +5168,15 @@
           <t xml:space="preserve">  DCF  (bear: FCF-15%)</t>
         </is>
       </c>
-      <c r="C28" s="52">
+      <c r="C28" s="53">
         <f>'DCF Valuation'!C26*0.78</f>
         <v/>
       </c>
-      <c r="D28" s="52">
+      <c r="D28" s="53">
         <f>'DCF Valuation'!C26*0.90</f>
         <v/>
       </c>
-      <c r="E28" s="52">
+      <c r="E28" s="53">
         <f>Assumptions!C7</f>
         <v/>
       </c>
@@ -4920,15 +5192,15 @@
           <t xml:space="preserve">  EV/EBITDA  (18-22x LTM)</t>
         </is>
       </c>
-      <c r="C29" s="52">
+      <c r="C29" s="53">
         <f>'Income Statement'!O13*18/Assumptions!E7</f>
         <v/>
       </c>
-      <c r="D29" s="52">
+      <c r="D29" s="53">
         <f>'Income Statement'!O13*22/Assumptions!E7</f>
         <v/>
       </c>
-      <c r="E29" s="52">
+      <c r="E29" s="53">
         <f>Assumptions!C7</f>
         <v/>
       </c>
@@ -4944,15 +5216,15 @@
           <t xml:space="preserve">  Current price  (mkt)</t>
         </is>
       </c>
-      <c r="C30" s="52">
+      <c r="C30" s="53">
         <f>Assumptions!C7</f>
         <v/>
       </c>
-      <c r="D30" s="52">
+      <c r="D30" s="53">
         <f>Assumptions!C7</f>
         <v/>
       </c>
-      <c r="E30" s="52">
+      <c r="E30" s="53">
         <f>Assumptions!C7</f>
         <v/>
       </c>
@@ -4996,4 +5268,821 @@
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="0070AD47"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:E24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="B1" s="20" t="inlineStr">
+        <is>
+          <t>SCENARIO ANALYSIS  -  Bear / Base / Bull</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="13" customHeight="1">
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Edit gold cells for Bear and Bull cases. Base links from Assumptions. Implied prices auto-calculate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="B4" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ASSUMPTION</t>
+        </is>
+      </c>
+      <c r="C4" s="63" t="inlineStr">
+        <is>
+          <t>BEAR</t>
+        </is>
+      </c>
+      <c r="D4" s="64" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="E4" s="65" t="inlineStr">
+        <is>
+          <t>BULL</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1">
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  REVENUE GROWTH</t>
+        </is>
+      </c>
+      <c r="C5" s="72" t="n"/>
+      <c r="D5" s="72" t="n"/>
+      <c r="E5" s="73" t="n"/>
+    </row>
+    <row r="6" ht="17" customHeight="1">
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Y1-Y5 Revenue Growth (avg)</t>
+        </is>
+      </c>
+      <c r="C6" s="21" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="D6" s="34">
+        <f>(Assumptions!C10+Assumptions!E10+Assumptions!C11+Assumptions!E11+Assumptions!C12)/5</f>
+        <v/>
+      </c>
+      <c r="E6" s="21" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="7" ht="17" customHeight="1">
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Y6-Y10 Revenue Growth (avg)</t>
+        </is>
+      </c>
+      <c r="C7" s="21" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="D7" s="34">
+        <f>(Assumptions!E12+Assumptions!C13+Assumptions!E13+Assumptions!C14+Assumptions!E14)/5</f>
+        <v/>
+      </c>
+      <c r="E7" s="21" t="n">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1">
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  MARGIN &amp; DISCOUNT RATE</t>
+        </is>
+      </c>
+      <c r="C8" s="72" t="n"/>
+      <c r="D8" s="72" t="n"/>
+      <c r="E8" s="73" t="n"/>
+    </row>
+    <row r="9" ht="17" customHeight="1">
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  EBITDA Margin %</t>
+        </is>
+      </c>
+      <c r="C9" s="21" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="D9" s="34">
+        <f>Assumptions!E16</f>
+        <v/>
+      </c>
+      <c r="E9" s="21" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="10" ht="17" customHeight="1">
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  FCF Margin (% of Revenue)</t>
+        </is>
+      </c>
+      <c r="C10" s="21" t="n">
+        <v>0.175</v>
+      </c>
+      <c r="D10" s="34">
+        <f>(Assumptions!E16-Assumptions!E17-Assumptions!C18+Assumptions!C19)*(1-Assumptions!E18)</f>
+        <v/>
+      </c>
+      <c r="E10" s="21" t="n">
+        <v>0.27</v>
+      </c>
+    </row>
+    <row r="11" ht="17" customHeight="1">
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  WACC</t>
+        </is>
+      </c>
+      <c r="C11" s="21" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="D11" s="34">
+        <f>WACC!E16</f>
+        <v/>
+      </c>
+      <c r="E11" s="21" t="n">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="12" ht="17" customHeight="1">
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Terminal Growth Rate</t>
+        </is>
+      </c>
+      <c r="C12" s="21" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="D12" s="34">
+        <f>Assumptions!C26</f>
+        <v/>
+      </c>
+      <c r="E12" s="21" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1">
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  COMMON INPUTS  (linked from model)</t>
+        </is>
+      </c>
+      <c r="C13" s="72" t="n"/>
+      <c r="D13" s="72" t="n"/>
+      <c r="E13" s="73" t="n"/>
+    </row>
+    <row r="14" ht="17" customHeight="1">
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Base Revenue Y0 ($M)</t>
+        </is>
+      </c>
+      <c r="C14" s="15">
+        <f>Assumptions!C28</f>
+        <v/>
+      </c>
+      <c r="D14" s="15">
+        <f>Assumptions!C28</f>
+        <v/>
+      </c>
+      <c r="E14" s="15">
+        <f>Assumptions!C28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="17" customHeight="1">
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Net Debt ($M)</t>
+        </is>
+      </c>
+      <c r="C15" s="15">
+        <f>Assumptions!C8-Assumptions!E8</f>
+        <v/>
+      </c>
+      <c r="D15" s="15">
+        <f>Assumptions!C8-Assumptions!E8</f>
+        <v/>
+      </c>
+      <c r="E15" s="15">
+        <f>Assumptions!C8-Assumptions!E8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="17" customHeight="1">
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Shares Outstanding (M)</t>
+        </is>
+      </c>
+      <c r="C16" s="15">
+        <f>Assumptions!E7</f>
+        <v/>
+      </c>
+      <c r="D16" s="15">
+        <f>Assumptions!E7</f>
+        <v/>
+      </c>
+      <c r="E16" s="15">
+        <f>Assumptions!E7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1">
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  VALUATION OUTPUT</t>
+        </is>
+      </c>
+      <c r="C17" s="72" t="n"/>
+      <c r="D17" s="72" t="n"/>
+      <c r="E17" s="73" t="n"/>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="B18" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  IMPLIED SHARE PRICE</t>
+        </is>
+      </c>
+      <c r="C18" s="66">
+        <f>IFERROR((SUMPRODUCT(C14*C10*(1+C6)^{1,2,3,4,5},1/(1+C11)^{1,2,3,4,5})+SUMPRODUCT(C14*C10*(1+C6)^5*(1+C7)^{1,2,3,4,5},1/(1+C11)^{6,7,8,9,10})+C14*C10*(1+C6)^5*(1+C7)^5*(1+C12)/MAX(C11-C12,0.0001)/(1+C11)^10-C15)/C16,"--")</f>
+        <v/>
+      </c>
+      <c r="D18" s="67">
+        <f>IFERROR((SUMPRODUCT(D14*D10*(1+D6)^{1,2,3,4,5},1/(1+D11)^{1,2,3,4,5})+SUMPRODUCT(D14*D10*(1+D6)^5*(1+D7)^{1,2,3,4,5},1/(1+D11)^{6,7,8,9,10})+D14*D10*(1+D6)^5*(1+D7)^5*(1+D12)/MAX(D11-D12,0.0001)/(1+D11)^10-D15)/D16,"--")</f>
+        <v/>
+      </c>
+      <c r="E18" s="68">
+        <f>IFERROR((SUMPRODUCT(E14*E10*(1+E6)^{1,2,3,4,5},1/(1+E11)^{1,2,3,4,5})+SUMPRODUCT(E14*E10*(1+E6)^5*(1+E7)^{1,2,3,4,5},1/(1+E11)^{6,7,8,9,10})+E14*E10*(1+E6)^5*(1+E7)^5*(1+E12)/MAX(E11-E12,0.0001)/(1+E11)^10-E15)/E16,"--")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="17" customHeight="1">
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Current Market Price ($)</t>
+        </is>
+      </c>
+      <c r="C19" s="53">
+        <f>Assumptions!C7</f>
+        <v/>
+      </c>
+      <c r="D19" s="53">
+        <f>Assumptions!C7</f>
+        <v/>
+      </c>
+      <c r="E19" s="53">
+        <f>Assumptions!C7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="17" customHeight="1">
+      <c r="B20" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Upside / (Downside) %</t>
+        </is>
+      </c>
+      <c r="C20" s="69">
+        <f>IFERROR((C18-D19)/D19,"--")</f>
+        <v/>
+      </c>
+      <c r="D20" s="54">
+        <f>IFERROR((D18-D19)/D19,"--")</f>
+        <v/>
+      </c>
+      <c r="E20" s="70">
+        <f>IFERROR((E18-D19)/D19,"--")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="15" customHeight="1">
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  EXPECTED VALUE SUMMARY</t>
+        </is>
+      </c>
+      <c r="C22" s="72" t="n"/>
+      <c r="D22" s="72" t="n"/>
+      <c r="E22" s="73" t="n"/>
+    </row>
+    <row r="23" ht="17" customHeight="1">
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Equal-Weighted Avg Price ($)</t>
+        </is>
+      </c>
+      <c r="C23" s="71">
+        <f>IFERROR((C18+D18+E18)/3,"--")</f>
+        <v/>
+      </c>
+      <c r="D23" s="72" t="n"/>
+      <c r="E23" s="73" t="n"/>
+    </row>
+    <row r="24" ht="17" customHeight="1">
+      <c r="B24" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Expected Upside / (Downside) %</t>
+        </is>
+      </c>
+      <c r="C24" s="24">
+        <f>IFERROR((C23-D19)/D19,"--")</f>
+        <v/>
+      </c>
+      <c r="D24" s="72" t="n"/>
+      <c r="E24" s="73" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="B17:E17"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="B13:E13"/>
+    <mergeCell ref="C23:E23"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B22:E22"/>
+    <mergeCell ref="C24:E24"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00833C00"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:K19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="B1" s="20" t="inlineStr">
+        <is>
+          <t>REVERSE DCF  -  Implied Growth Rate at Current Price</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="13" customHeight="1">
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Find the column where implied price = current market price. That growth rate is what the market is pricing in.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="17" customHeight="1">
+      <c r="B4" s="74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Target / Market Price ($)</t>
+        </is>
+      </c>
+      <c r="C4" s="73" t="n"/>
+      <c r="D4" s="10">
+        <f>Assumptions!C7</f>
+        <v/>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Edit D4 to test any price. Green = implied price &gt;= D4 (potential buy).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="17" customHeight="1">
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  FCF Margin (model-derived)</t>
+        </is>
+      </c>
+      <c r="C5" s="73" t="n"/>
+      <c r="D5" s="34">
+        <f>(Assumptions!E16-Assumptions!E17-Assumptions!C18+Assumptions!C19)*(1-Assumptions!E18)</f>
+        <v/>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Flows from Assumptions — edit margins there to see impact here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="17" customHeight="1">
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Terminal Growth Rate</t>
+        </is>
+      </c>
+      <c r="C6" s="73" t="n"/>
+      <c r="D6" s="34">
+        <f>'DCF Valuation'!C5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  TABLE: Implied Share Price by Uniform Revenue Growth Rate x WACC -- find where implied price = market price</t>
+        </is>
+      </c>
+      <c r="C8" s="72" t="n"/>
+      <c r="D8" s="72" t="n"/>
+      <c r="E8" s="72" t="n"/>
+      <c r="F8" s="72" t="n"/>
+      <c r="G8" s="72" t="n"/>
+      <c r="H8" s="72" t="n"/>
+      <c r="I8" s="72" t="n"/>
+      <c r="J8" s="73" t="n"/>
+    </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="B9" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  WACC \ Growth</t>
+        </is>
+      </c>
+      <c r="C9" s="75" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="D9" s="75" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="E9" s="75" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="F9" s="75" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="G9" s="75" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H9" s="75" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="I9" s="75" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J9" s="75" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="10" ht="17" customHeight="1">
+      <c r="B10" s="59">
+        <f>'DCF Valuation'!C4+(-0.015)</f>
+        <v/>
+      </c>
+      <c r="C10" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+C9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B10)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+C9)^10*(1+D6)/MAX(B10-D6,0.0001)/(1+B10)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="D10" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+D9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B10)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+D9)^10*(1+D6)/MAX(B10-D6,0.0001)/(1+B10)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="E10" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+E9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B10)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+E9)^10*(1+D6)/MAX(B10-D6,0.0001)/(1+B10)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="F10" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+F9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B10)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+F9)^10*(1+D6)/MAX(B10-D6,0.0001)/(1+B10)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="G10" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+G9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B10)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+G9)^10*(1+D6)/MAX(B10-D6,0.0001)/(1+B10)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="H10" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+H9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B10)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+H9)^10*(1+D6)/MAX(B10-D6,0.0001)/(1+B10)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="I10" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+I9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B10)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+I9)^10*(1+D6)/MAX(B10-D6,0.0001)/(1+B10)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="J10" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+J9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B10)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+J9)^10*(1+D6)/MAX(B10-D6,0.0001)/(1+B10)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="17" customHeight="1">
+      <c r="B11" s="59">
+        <f>'DCF Valuation'!C4+(-0.01)</f>
+        <v/>
+      </c>
+      <c r="C11" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+C9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B11)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+C9)^10*(1+D6)/MAX(B11-D6,0.0001)/(1+B11)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="D11" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+D9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B11)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+D9)^10*(1+D6)/MAX(B11-D6,0.0001)/(1+B11)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="E11" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+E9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B11)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+E9)^10*(1+D6)/MAX(B11-D6,0.0001)/(1+B11)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="F11" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+F9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B11)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+F9)^10*(1+D6)/MAX(B11-D6,0.0001)/(1+B11)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="G11" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+G9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B11)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+G9)^10*(1+D6)/MAX(B11-D6,0.0001)/(1+B11)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="H11" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+H9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B11)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+H9)^10*(1+D6)/MAX(B11-D6,0.0001)/(1+B11)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="I11" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+I9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B11)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+I9)^10*(1+D6)/MAX(B11-D6,0.0001)/(1+B11)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="J11" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+J9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B11)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+J9)^10*(1+D6)/MAX(B11-D6,0.0001)/(1+B11)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="17" customHeight="1">
+      <c r="B12" s="59">
+        <f>'DCF Valuation'!C4+(-0.005)</f>
+        <v/>
+      </c>
+      <c r="C12" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+C9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B12)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+C9)^10*(1+D6)/MAX(B12-D6,0.0001)/(1+B12)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="D12" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+D9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B12)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+D9)^10*(1+D6)/MAX(B12-D6,0.0001)/(1+B12)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="E12" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+E9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B12)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+E9)^10*(1+D6)/MAX(B12-D6,0.0001)/(1+B12)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="F12" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+F9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B12)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+F9)^10*(1+D6)/MAX(B12-D6,0.0001)/(1+B12)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="G12" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+G9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B12)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+G9)^10*(1+D6)/MAX(B12-D6,0.0001)/(1+B12)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="H12" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+H9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B12)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+H9)^10*(1+D6)/MAX(B12-D6,0.0001)/(1+B12)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="I12" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+I9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B12)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+I9)^10*(1+D6)/MAX(B12-D6,0.0001)/(1+B12)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="J12" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+J9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B12)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+J9)^10*(1+D6)/MAX(B12-D6,0.0001)/(1+B12)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="17" customHeight="1">
+      <c r="B13" s="59">
+        <f>'DCF Valuation'!C4+(0.0)</f>
+        <v/>
+      </c>
+      <c r="C13" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+C9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B13)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+C9)^10*(1+D6)/MAX(B13-D6,0.0001)/(1+B13)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="D13" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+D9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B13)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+D9)^10*(1+D6)/MAX(B13-D6,0.0001)/(1+B13)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="E13" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+E9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B13)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+E9)^10*(1+D6)/MAX(B13-D6,0.0001)/(1+B13)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="F13" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+F9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B13)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+F9)^10*(1+D6)/MAX(B13-D6,0.0001)/(1+B13)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="G13" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+G9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B13)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+G9)^10*(1+D6)/MAX(B13-D6,0.0001)/(1+B13)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="H13" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+H9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B13)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+H9)^10*(1+D6)/MAX(B13-D6,0.0001)/(1+B13)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="I13" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+I9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B13)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+I9)^10*(1+D6)/MAX(B13-D6,0.0001)/(1+B13)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="J13" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+J9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B13)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+J9)^10*(1+D6)/MAX(B13-D6,0.0001)/(1+B13)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="17" customHeight="1">
+      <c r="B14" s="59">
+        <f>'DCF Valuation'!C4+(0.005)</f>
+        <v/>
+      </c>
+      <c r="C14" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+C9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B14)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+C9)^10*(1+D6)/MAX(B14-D6,0.0001)/(1+B14)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="D14" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+D9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B14)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+D9)^10*(1+D6)/MAX(B14-D6,0.0001)/(1+B14)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="E14" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+E9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B14)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+E9)^10*(1+D6)/MAX(B14-D6,0.0001)/(1+B14)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="F14" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+F9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B14)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+F9)^10*(1+D6)/MAX(B14-D6,0.0001)/(1+B14)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="G14" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+G9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B14)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+G9)^10*(1+D6)/MAX(B14-D6,0.0001)/(1+B14)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="H14" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+H9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B14)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+H9)^10*(1+D6)/MAX(B14-D6,0.0001)/(1+B14)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="I14" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+I9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B14)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+I9)^10*(1+D6)/MAX(B14-D6,0.0001)/(1+B14)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="J14" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+J9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B14)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+J9)^10*(1+D6)/MAX(B14-D6,0.0001)/(1+B14)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="17" customHeight="1">
+      <c r="B15" s="59">
+        <f>'DCF Valuation'!C4+(0.01)</f>
+        <v/>
+      </c>
+      <c r="C15" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+C9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B15)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+C9)^10*(1+D6)/MAX(B15-D6,0.0001)/(1+B15)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="D15" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+D9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B15)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+D9)^10*(1+D6)/MAX(B15-D6,0.0001)/(1+B15)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="E15" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+E9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B15)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+E9)^10*(1+D6)/MAX(B15-D6,0.0001)/(1+B15)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="F15" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+F9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B15)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+F9)^10*(1+D6)/MAX(B15-D6,0.0001)/(1+B15)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="G15" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+G9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B15)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+G9)^10*(1+D6)/MAX(B15-D6,0.0001)/(1+B15)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="H15" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+H9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B15)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+H9)^10*(1+D6)/MAX(B15-D6,0.0001)/(1+B15)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="I15" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+I9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B15)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+I9)^10*(1+D6)/MAX(B15-D6,0.0001)/(1+B15)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="J15" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+J9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B15)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+J9)^10*(1+D6)/MAX(B15-D6,0.0001)/(1+B15)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="17" customHeight="1">
+      <c r="B16" s="59">
+        <f>'DCF Valuation'!C4+(0.015)</f>
+        <v/>
+      </c>
+      <c r="C16" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+C9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B16)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+C9)^10*(1+D6)/MAX(B16-D6,0.0001)/(1+B16)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="D16" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+D9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B16)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+D9)^10*(1+D6)/MAX(B16-D6,0.0001)/(1+B16)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="E16" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+E9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B16)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+E9)^10*(1+D6)/MAX(B16-D6,0.0001)/(1+B16)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="F16" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+F9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B16)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+F9)^10*(1+D6)/MAX(B16-D6,0.0001)/(1+B16)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="G16" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+G9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B16)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+G9)^10*(1+D6)/MAX(B16-D6,0.0001)/(1+B16)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="H16" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+H9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B16)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+H9)^10*(1+D6)/MAX(B16-D6,0.0001)/(1+B16)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="I16" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+I9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B16)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+I9)^10*(1+D6)/MAX(B16-D6,0.0001)/(1+B16)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+      <c r="J16" s="53">
+        <f>IFERROR((SUMPRODUCT(Assumptions!C28*D5*(1+J9)^{1,2,3,4,5,6,7,8,9,10},1/(1+B16)^{1,2,3,4,5,6,7,8,9,10})+Assumptions!C28*D5*(1+J9)^10*(1+D6)/MAX(B16-D6,0.0001)/(1+B16)^10-(Assumptions!C8-Assumptions!E8))/Assumptions!E7,"--")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="14" customHeight="1">
+      <c r="B18" s="76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  HOW TO READ: Find your WACC row (0.00% offset = model WACC). Scan right to find where implied price matches market price. That column = market-implied growth rate.</t>
+        </is>
+      </c>
+      <c r="C18" s="72" t="n"/>
+      <c r="D18" s="72" t="n"/>
+      <c r="E18" s="72" t="n"/>
+      <c r="F18" s="72" t="n"/>
+      <c r="G18" s="72" t="n"/>
+      <c r="H18" s="72" t="n"/>
+      <c r="I18" s="72" t="n"/>
+      <c r="J18" s="72" t="n"/>
+      <c r="K18" s="73" t="n"/>
+    </row>
+    <row r="19" ht="14" customHeight="1">
+      <c r="B19" s="76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  This uses a UNIFORM growth rate for all 10 years. For two-phase growth analysis, see the Scenarios sheet.</t>
+        </is>
+      </c>
+      <c r="C19" s="72" t="n"/>
+      <c r="D19" s="72" t="n"/>
+      <c r="E19" s="72" t="n"/>
+      <c r="F19" s="72" t="n"/>
+      <c r="G19" s="72" t="n"/>
+      <c r="H19" s="72" t="n"/>
+      <c r="I19" s="72" t="n"/>
+      <c r="J19" s="72" t="n"/>
+      <c r="K19" s="73" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="E5:K5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B1:K1"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B18:K18"/>
+    <mergeCell ref="E4:K4"/>
+    <mergeCell ref="B8:J8"/>
+    <mergeCell ref="B2:K2"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B19:K19"/>
+  </mergeCells>
+  <conditionalFormatting sqref="C10:J16">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00FFC7CE"/>
+        <color rgb="00FFEB9C"/>
+        <color rgb="00C6EFCE"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>